<commit_message>
docs(xlsx): HELIX Dashboards sheet — add Shopify, Mailchimp, HELIX OPS (A/B) connectors
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCTS/HELIX-external-connections.xlsx
+++ b/PRODUCTS/HELIX-external-connections.xlsx
@@ -8125,7 +8125,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8609,6 +8609,105 @@
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Shopify</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Data source</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>E-commerce metrics into dashboards (sales / orders / AOV)</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Shopify Admin API token + shop domain (connector, encrypted via SECRETS_KEY)</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>&lt;shop&gt;.myshopify.com → Admin API</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Mailchimp</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Data source</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Email list metrics (subscribers / unsubscribes)</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Mailchimp API key (connector, encrypted)</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>mailchimp.com → Account → API keys</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>HELIX OPS (campaign A/B)</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Data source / cross-product</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Pull campaign A/B metrics (impressions/views/clicks/variants per channel) into dashboards</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>base_url + Export Secret + OPS workspace id (connector)</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>internal (helix-ops /api/export/campaign-metrics)</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
docs: dashboards connectors 9 (+Rav-Messer +ActiveTrail) in doc + xlsx
</commit_message>
<xml_diff>
--- a/PRODUCTS/HELIX-external-connections.xlsx
+++ b/PRODUCTS/HELIX-external-connections.xlsx
@@ -8125,7 +8125,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8708,6 +8708,80 @@
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Rav-Messer (Responder)</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Data source</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Israeli email/SMS marketing metrics (list subscribers) into dashboards</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>User Key (+ optional Secret) — connector, encrypted</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>support@responder.co.il / 03-717-7777</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>🔧 Code ready</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>verify endpoint schema</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>ActiveTrail</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Data source</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Israeli email/SMS marketing metrics (contacts/subscribers) into dashboards</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>API key (connector, encrypted)</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>ActiveTrail account → Settings → API</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>🔧 Code ready</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>verify endpoint schema</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
docs: add InforU connector (doc + xlsx)
</commit_message>
<xml_diff>
--- a/PRODUCTS/HELIX-external-connections.xlsx
+++ b/PRODUCTS/HELIX-external-connections.xlsx
@@ -8125,7 +8125,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8778,6 +8778,43 @@
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>verify endpoint schema</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>InforU</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Data source</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Israeli SMS/email marketing metrics (contact groups) into dashboards</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>API key (connector, encrypted)</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>InforU account → API</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>🔧 Code ready</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
         <is>
           <t>verify endpoint schema</t>
         </is>

</xml_diff>

<commit_message>
docs: Growth Doctor — bot+dashboard integration, build-status, xlsx sheet+master
</commit_message>
<xml_diff>
--- a/PRODUCTS/HELIX-external-connections.xlsx
+++ b/PRODUCTS/HELIX-external-connections.xlsx
@@ -17,6 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Channels matrix" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shared accounts" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup order" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HELIX Growth Doctor" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -636,7 +637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G113"/>
+  <dimension ref="A1:G130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3994,6 +3995,512 @@
         </is>
       </c>
       <c r="G113" s="7" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="15" t="inlineStr">
+        <is>
+          <t>HELIX Growth Doctor (Product 07)</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="4" t="inlineStr">
+        <is>
+          <t>Service / Channel</t>
+        </is>
+      </c>
+      <c r="B116" s="4" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C116" s="4" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="D116" s="4" t="inlineStr">
+        <is>
+          <t>Connect (token / OAuth / webhook / env)</t>
+        </is>
+      </c>
+      <c r="E116" s="4" t="inlineStr">
+        <is>
+          <t>Where to get it</t>
+        </is>
+      </c>
+      <c r="F116" s="4" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G116" s="4" t="inlineStr">
+        <is>
+          <t>Connected?</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="5" t="inlineStr">
+        <is>
+          <t>Supabase</t>
+        </is>
+      </c>
+      <c r="B117" s="5" t="inlineStr">
+        <is>
+          <t>Core / DB</t>
+        </is>
+      </c>
+      <c r="C117" s="5" t="inlineStr">
+        <is>
+          <t>Events (funnel/returns) + cohorts + insights + Auth + RLS</t>
+        </is>
+      </c>
+      <c r="D117" s="5" t="inlineStr">
+        <is>
+          <t>NEXT_PUBLIC_SUPABASE_URL / _ANON_KEY / SUPABASE_SERVICE_ROLE_KEY</t>
+        </is>
+      </c>
+      <c r="E117" s="5" t="inlineStr">
+        <is>
+          <t>supabase.com</t>
+        </is>
+      </c>
+      <c r="F117" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G117" s="7" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="5" t="inlineStr">
+        <is>
+          <t>Anthropic Claude</t>
+        </is>
+      </c>
+      <c r="B118" s="5" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="C118" s="5" t="inlineStr">
+        <is>
+          <t>Insight quality tier (recommendation copy)</t>
+        </is>
+      </c>
+      <c r="D118" s="5" t="inlineStr">
+        <is>
+          <t>ANTHROPIC_API_KEY (+ CONTENT_MODEL)</t>
+        </is>
+      </c>
+      <c r="E118" s="5" t="inlineStr">
+        <is>
+          <t>console.anthropic.com</t>
+        </is>
+      </c>
+      <c r="F118" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G118" s="7" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="5" t="inlineStr">
+        <is>
+          <t>Ollama</t>
+        </is>
+      </c>
+      <c r="B119" s="5" t="inlineStr">
+        <is>
+          <t>AI / local</t>
+        </is>
+      </c>
+      <c r="C119" s="5" t="inlineStr">
+        <is>
+          <t>CRO agent runs on-prem — privacy (data stays with business)</t>
+        </is>
+      </c>
+      <c r="D119" s="5" t="inlineStr">
+        <is>
+          <t>OLLAMA_BASE_URL / OLLAMA_MODEL</t>
+        </is>
+      </c>
+      <c r="E119" s="5" t="inlineStr">
+        <is>
+          <t>ollama.com</t>
+        </is>
+      </c>
+      <c r="F119" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G119" s="7" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="5" t="inlineStr">
+        <is>
+          <t>HELIX tag (JS snippet)</t>
+        </is>
+      </c>
+      <c r="B120" s="5" t="inlineStr">
+        <is>
+          <t>Data source</t>
+        </is>
+      </c>
+      <c r="C120" s="5" t="inlineStr">
+        <is>
+          <t>First-party funnel + return events (embed on site)</t>
+        </is>
+      </c>
+      <c r="D120" s="5" t="inlineStr">
+        <is>
+          <t>public/helix-tag.js -&gt; /api/collect</t>
+        </is>
+      </c>
+      <c r="E120" s="5" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F120" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G120" s="7" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="5" t="inlineStr">
+        <is>
+          <t>Microsoft Clarity</t>
+        </is>
+      </c>
+      <c r="B121" s="5" t="inlineStr">
+        <is>
+          <t>Data source</t>
+        </is>
+      </c>
+      <c r="C121" s="5" t="inlineStr">
+        <is>
+          <t>Heatmaps / session replay / funnels (FREE)</t>
+        </is>
+      </c>
+      <c r="D121" s="5" t="inlineStr">
+        <is>
+          <t>Clarity API token (connector)</t>
+        </is>
+      </c>
+      <c r="E121" s="5" t="inlineStr">
+        <is>
+          <t>clarity.microsoft.com</t>
+        </is>
+      </c>
+      <c r="F121" s="6" t="inlineStr">
+        <is>
+          <t>🔧 Planned</t>
+        </is>
+      </c>
+      <c r="G121" s="7" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="5" t="inlineStr">
+        <is>
+          <t>Google Analytics (GA4)</t>
+        </is>
+      </c>
+      <c r="B122" s="5" t="inlineStr">
+        <is>
+          <t>Data source</t>
+        </is>
+      </c>
+      <c r="C122" s="5" t="inlineStr">
+        <is>
+          <t>Traffic + conversion metrics</t>
+        </is>
+      </c>
+      <c r="D122" s="5" t="inlineStr">
+        <is>
+          <t>GOOGLE_OAUTH_* (reuse dashboards)</t>
+        </is>
+      </c>
+      <c r="E122" s="5" t="inlineStr">
+        <is>
+          <t>console.cloud.google.com</t>
+        </is>
+      </c>
+      <c r="F122" s="6" t="inlineStr">
+        <is>
+          <t>🔧 Planned</t>
+        </is>
+      </c>
+      <c r="G122" s="7" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="5" t="inlineStr">
+        <is>
+          <t>Mixpanel / Amplitude / PostHog</t>
+        </is>
+      </c>
+      <c r="B123" s="5" t="inlineStr">
+        <is>
+          <t>Data source</t>
+        </is>
+      </c>
+      <c r="C123" s="5" t="inlineStr">
+        <is>
+          <t>Retention / cohorts (optional, BYO)</t>
+        </is>
+      </c>
+      <c r="D123" s="5" t="inlineStr">
+        <is>
+          <t>API key per tool (connector)</t>
+        </is>
+      </c>
+      <c r="E123" s="5" t="inlineStr">
+        <is>
+          <t>each tool</t>
+        </is>
+      </c>
+      <c r="F123" s="6" t="inlineStr">
+        <is>
+          <t>⚪ BYO</t>
+        </is>
+      </c>
+      <c r="G123" s="7" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="5" t="inlineStr">
+        <is>
+          <t>WhatsApp Cloud API</t>
+        </is>
+      </c>
+      <c r="B124" s="5" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="C124" s="5" t="inlineStr">
+        <is>
+          <t>Doctor digest + inbound actions</t>
+        </is>
+      </c>
+      <c r="D124" s="5" t="inlineStr">
+        <is>
+          <t>WHATSAPP_TOKEN / WHATSAPP_PHONE_ID</t>
+        </is>
+      </c>
+      <c r="E124" s="5" t="inlineStr">
+        <is>
+          <t>developers.facebook.com</t>
+        </is>
+      </c>
+      <c r="F124" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G124" s="7" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="5" t="inlineStr">
+        <is>
+          <t>Telegram Bot</t>
+        </is>
+      </c>
+      <c r="B125" s="5" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="C125" s="5" t="inlineStr">
+        <is>
+          <t>Doctor digest + inbound actions (/api/bot)</t>
+        </is>
+      </c>
+      <c r="D125" s="5" t="inlineStr">
+        <is>
+          <t>TELEGRAM_BOT_TOKEN</t>
+        </is>
+      </c>
+      <c r="E125" s="5" t="inlineStr">
+        <is>
+          <t>@BotFather</t>
+        </is>
+      </c>
+      <c r="F125" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G125" s="7" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="5" t="inlineStr">
+        <is>
+          <t>Email (Resend)</t>
+        </is>
+      </c>
+      <c r="B126" s="5" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="C126" s="5" t="inlineStr">
+        <is>
+          <t>Digest / report delivery</t>
+        </is>
+      </c>
+      <c r="D126" s="5" t="inlineStr">
+        <is>
+          <t>RESEND_API_KEY / EMAIL_FROM</t>
+        </is>
+      </c>
+      <c r="E126" s="5" t="inlineStr">
+        <is>
+          <t>resend.com</t>
+        </is>
+      </c>
+      <c r="F126" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G126" s="7" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="5" t="inlineStr">
+        <is>
+          <t>HELIX OPS (reuse)</t>
+        </is>
+      </c>
+      <c r="B127" s="5" t="inlineStr">
+        <is>
+          <t>Cross-product</t>
+        </is>
+      </c>
+      <c r="C127" s="5" t="inlineStr">
+        <is>
+          <t>Execute the FIX — Landing / A-B / Campaigns / win-back</t>
+        </is>
+      </c>
+      <c r="D127" s="5" t="inlineStr">
+        <is>
+          <t>internal (same ecosystem)</t>
+        </is>
+      </c>
+      <c r="E127" s="5" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F127" s="6" t="inlineStr">
+        <is>
+          <t>🔧 Planned</t>
+        </is>
+      </c>
+      <c r="G127" s="7" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="5" t="inlineStr">
+        <is>
+          <t>HELIX DASHBOARDS export</t>
+        </is>
+      </c>
+      <c r="B128" s="5" t="inlineStr">
+        <is>
+          <t>Cross-product</t>
+        </is>
+      </c>
+      <c r="C128" s="5" t="inlineStr">
+        <is>
+          <t>Push CRO/funnel/retention metrics to super-dashboard</t>
+        </is>
+      </c>
+      <c r="D128" s="5" t="inlineStr">
+        <is>
+          <t>EXPORT_SECRET (/api/export/growth-metrics)</t>
+        </is>
+      </c>
+      <c r="E128" s="5" t="inlineStr">
+        <is>
+          <t>self-chosen</t>
+        </is>
+      </c>
+      <c r="F128" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G128" s="7" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="5" t="inlineStr">
+        <is>
+          <t>Cron secret</t>
+        </is>
+      </c>
+      <c r="B129" s="5" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="C129" s="5" t="inlineStr">
+        <is>
+          <t>Autonomous loop (measure-&gt;fix-&gt;re-measure)</t>
+        </is>
+      </c>
+      <c r="D129" s="5" t="inlineStr">
+        <is>
+          <t>CRON_SECRET</t>
+        </is>
+      </c>
+      <c r="E129" s="5" t="inlineStr">
+        <is>
+          <t>self-chosen</t>
+        </is>
+      </c>
+      <c r="F129" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G129" s="7" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="5" t="inlineStr">
+        <is>
+          <t>Vercel</t>
+        </is>
+      </c>
+      <c r="B130" s="5" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="C130" s="5" t="inlineStr">
+        <is>
+          <t>Hosting + Cron</t>
+        </is>
+      </c>
+      <c r="D130" s="5" t="inlineStr">
+        <is>
+          <t>git push (repo TBD)</t>
+        </is>
+      </c>
+      <c r="E130" s="5" t="inlineStr">
+        <is>
+          <t>vercel.com</t>
+        </is>
+      </c>
+      <c r="F130" s="6" t="inlineStr">
+        <is>
+          <t>✅ Core</t>
+        </is>
+      </c>
+      <c r="G130" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -4824,6 +5331,535 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>HELIX Growth Doctor (Product 07)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Service / Channel</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Connect (token / OAuth / webhook / env)</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>Where to get it</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>Connected?</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Supabase</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Core / DB</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Events (funnel/returns) + cohorts + insights + Auth + RLS</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>NEXT_PUBLIC_SUPABASE_URL / _ANON_KEY / SUPABASE_SERVICE_ROLE_KEY</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>supabase.com</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Anthropic Claude</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Insight quality tier (recommendation copy)</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>ANTHROPIC_API_KEY (+ CONTENT_MODEL)</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>console.anthropic.com</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Ollama</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>AI / local</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>CRO agent runs on-prem — privacy (data stays with business)</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>OLLAMA_BASE_URL / OLLAMA_MODEL</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>ollama.com</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>HELIX tag (JS snippet)</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Data source</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>First-party funnel + return events (embed on site)</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>public/helix-tag.js -&gt; /api/collect</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Microsoft Clarity</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Data source</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Heatmaps / session replay / funnels (FREE)</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Clarity API token (connector)</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>clarity.microsoft.com</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>🔧 Planned</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Google Analytics (GA4)</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Data source</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Traffic + conversion metrics</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>GOOGLE_OAUTH_* (reuse dashboards)</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>console.cloud.google.com</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>🔧 Planned</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Mixpanel / Amplitude / PostHog</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Data source</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Retention / cohorts (optional, BYO)</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>API key per tool (connector)</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>each tool</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>⚪ BYO</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>WhatsApp Cloud API</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Doctor digest + inbound actions</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>WHATSAPP_TOKEN / WHATSAPP_PHONE_ID</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>developers.facebook.com</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Telegram Bot</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Doctor digest + inbound actions (/api/bot)</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>TELEGRAM_BOT_TOKEN</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>@BotFather</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Email (Resend)</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Digest / report delivery</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>RESEND_API_KEY / EMAIL_FROM</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>resend.com</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>HELIX OPS (reuse)</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Cross-product</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Execute the FIX — Landing / A-B / Campaigns / win-back</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>internal (same ecosystem)</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>🔧 Planned</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>HELIX DASHBOARDS export</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Cross-product</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Push CRO/funnel/retention metrics to super-dashboard</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>EXPORT_SECRET (/api/export/growth-metrics)</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>self-chosen</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Cron secret</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Autonomous loop (measure-&gt;fix-&gt;re-measure)</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>CRON_SECRET</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>self-chosen</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Vercel</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Hosting + Cron</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>git push (repo TBD)</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>vercel.com</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>✅ Core</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
docs(growth-doctor): update build-status §11 to built MVP + xlsx repo name
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCTS/HELIX-external-connections.xlsx
+++ b/PRODUCTS/HELIX-external-connections.xlsx
@@ -663,6 +663,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1301,6 +1302,7 @@
       </c>
       <c r="G23" s="7" t="inlineStr"/>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="10" t="inlineStr">
         <is>
@@ -2005,6 +2007,7 @@
       </c>
       <c r="G46" s="7" t="inlineStr"/>
     </row>
+    <row r="47"/>
     <row r="48">
       <c r="A48" s="12" t="inlineStr">
         <is>
@@ -2577,6 +2580,7 @@
       </c>
       <c r="G65" s="7" t="inlineStr"/>
     </row>
+    <row r="66"/>
     <row r="67">
       <c r="A67" s="13" t="inlineStr">
         <is>
@@ -3314,6 +3318,7 @@
       </c>
       <c r="G89" s="7" t="inlineStr"/>
     </row>
+    <row r="90"/>
     <row r="91">
       <c r="A91" s="14" t="inlineStr">
         <is>
@@ -3523,6 +3528,7 @@
       </c>
       <c r="G97" s="7" t="inlineStr"/>
     </row>
+    <row r="98"/>
     <row r="99">
       <c r="A99" s="15" t="inlineStr">
         <is>
@@ -3996,6 +4002,7 @@
       </c>
       <c r="G113" s="7" t="inlineStr"/>
     </row>
+    <row r="114"/>
     <row r="115">
       <c r="A115" s="15" t="inlineStr">
         <is>
@@ -4487,7 +4494,7 @@
       </c>
       <c r="D130" s="5" t="inlineStr">
         <is>
-          <t>git push (repo TBD)</t>
+          <t>git push (Helix-growth-doctor)</t>
         </is>
       </c>
       <c r="E130" s="5" t="inlineStr">
@@ -5840,7 +5847,7 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>git push (repo TBD)</t>
+          <t>git push (Helix-growth-doctor)</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">

</xml_diff>

<commit_message>
docs(sdr): add §3.6 Lifecycle & Reminders engine — spec + data model + Excel connections
- §3.6: appointment/renewal/replenishment/birthday reminders, coupons, import
- data model: lifecycle_customers/appointments/purchases/coupons/lifecycle_jobs
- Excel SDR sheet: WhatsApp templates (proactive gap), lifecycle cron, import
- regenerated .docx

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCTS/HELIX-external-connections.xlsx
+++ b/PRODUCTS/HELIX-external-connections.xlsx
@@ -663,7 +663,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1302,7 +1301,6 @@
       </c>
       <c r="G23" s="7" t="inlineStr"/>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="A25" s="10" t="inlineStr">
         <is>
@@ -2007,7 +2005,6 @@
       </c>
       <c r="G46" s="7" t="inlineStr"/>
     </row>
-    <row r="47"/>
     <row r="48">
       <c r="A48" s="12" t="inlineStr">
         <is>
@@ -2580,7 +2577,6 @@
       </c>
       <c r="G65" s="7" t="inlineStr"/>
     </row>
-    <row r="66"/>
     <row r="67">
       <c r="A67" s="13" t="inlineStr">
         <is>
@@ -3318,7 +3314,6 @@
       </c>
       <c r="G89" s="7" t="inlineStr"/>
     </row>
-    <row r="90"/>
     <row r="91">
       <c r="A91" s="14" t="inlineStr">
         <is>
@@ -3528,7 +3523,6 @@
       </c>
       <c r="G97" s="7" t="inlineStr"/>
     </row>
-    <row r="98"/>
     <row r="99">
       <c r="A99" s="15" t="inlineStr">
         <is>
@@ -4002,7 +3996,6 @@
       </c>
       <c r="G113" s="7" t="inlineStr"/>
     </row>
-    <row r="114"/>
     <row r="115">
       <c r="A115" s="15" t="inlineStr">
         <is>
@@ -5873,7 +5866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6470,7 +6463,7 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Executor cron gate + approve links + inbound routing</t>
+          <t>Executor + lifecycle cron gate + approve/confirm-cancel links + inbound routing</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
@@ -6522,6 +6515,105 @@
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>WhatsApp Message Templates</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Channel / §3.6</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Proactive lifecycle reminders (appt/renewal/replenish/birthday) OUTSIDE 24h window require APPROVED templates</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Meta WhatsApp Manager → Message Templates (per lang, category=UTILITY/MARKETING)</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>business.facebook.com → WhatsApp Manager</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>🔧 Needed for §3.6 proactive send</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Lifecycle Cron</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Infra / §3.6</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Send due reminder jobs every ~15 min (lifecycle_jobs → WhatsApp)</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>GET /api/lifecycle/cron?secret=EXECUTOR_SECRET (Vercel Cron)</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>vercel.json crons</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Customer Import</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Data / §3.6</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Bulk-load existing customers (personal + pet/secondary entity) from Excel/registration; auto-schedules birthdays</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>POST /api/lifecycle/import (CSV or JSON)</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>n/a (internal)</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
docs(sdr): document §3.6.1 WhatsApp templates, §3.6.2 operator commands, §3.6.3 metrics export
- template catalog table (8 approved templates) + sync route + fallback flow
- operator bot commands table + bot_links identity
- sdr-metrics export endpoint + helix_sdr connector
- Excel: template sync / operator commands / metrics export rows; dashboards export ready

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCTS/HELIX-external-connections.xlsx
+++ b/PRODUCTS/HELIX-external-connections.xlsx
@@ -5866,7 +5866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6445,7 +6445,7 @@
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>🔧 Planned</t>
+          <t>✅ Export ready (connector pull)</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr"/>
@@ -6614,6 +6614,105 @@
         </is>
       </c>
       <c r="G23" s="7" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Template Sync</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Infra / §3.6.1</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Register all WhatsApp templates on the WABA (idempotent)</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>POST /api/templates/sync?secret=EXECUTOR_SECRET (needs waba_id in channel config)</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>n/a (internal)</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Operator Bot Commands</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Bot / §3.6.2</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Run schedule/import/stats from WhatsApp/Telegram in free Hebrew (bot_links identity)</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>bot_links table + LLM parse (Haiku); wired into telegram/whatsapp webhooks</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>n/a (internal)</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>SDR Metrics Export</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Infra / §3.6.3</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Pull endpoint for HELIX Dashboards connector helix_sdr</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>GET /api/export/sdr-metrics?workspace=&amp;secret=EXPORT_SECRET</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>n/a (internal)</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
docs(sdr): §3.6.4 OTP + order-status + quick-reply templates
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCTS/HELIX-external-connections.xlsx
+++ b/PRODUCTS/HELIX-external-connections.xlsx
@@ -5866,7 +5866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6713,6 +6713,105 @@
         </is>
       </c>
       <c r="G26" s="7" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>WhatsApp OTP (AUTHENTICATION)</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Auth / §3.6.4</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Customer OTP verification via approved AUTHENTICATION template</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>sdr_otp template (needs Meta AUTHENTICATION approval); POST /api/auth/otp</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>WhatsApp Manager</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>🔧 Needs Meta approval</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Order Status Updates</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Commerce / §3.6.4</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>order_confirmed/shipped/ready templates</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>POST /api/lifecycle/order-status; business system supplies order data</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>n/a (internal)</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Quick-Reply Buttons</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Bot / §3.6.4</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>One-tap confirm/cancel/reorder via template quick_reply payloads</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>handled in whatsapp webhook (applyButtonAction)</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>n/a (internal)</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
docs(sdr): §3.6.5 inbound replies — canned/quick replies, Messenger wiring, bot access
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCTS/HELIX-external-connections.xlsx
+++ b/PRODUCTS/HELIX-external-connections.xlsx
@@ -5866,7 +5866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6181,7 +6181,7 @@
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>🔧 Planned</t>
+          <t>✅ Wired (§3.6.5)</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr"/>
@@ -6812,6 +6812,72 @@
         </is>
       </c>
       <c r="G29" s="7" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Messenger (Facebook)</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Channel / §3.6.5</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Inbound Page DM auto-reply via existing AI engine</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Meta app + Page access_token + META_VERIFY_TOKEN; /api/webhooks/messenger</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>developers.facebook.com → Messenger</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired (§3.6.5)</t>
+        </is>
+      </c>
+      <c r="G30" s="7" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Canned / Quick Replies</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Inbound / §3.6.5</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Instant FAQ answers to common inquiries (in-window, no Meta approval)</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>canned_replies table + lib/canned; matched before AI draft</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>n/a (internal)</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
docs(sdr): §3.6.6 LinkedIn inbound + cold-email templates
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCTS/HELIX-external-connections.xlsx
+++ b/PRODUCTS/HELIX-external-connections.xlsx
@@ -5866,7 +5866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6247,7 +6247,7 @@
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>🔧 Planned</t>
+          <t>✅ Inbound wired (§3.6.6); send via extension</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr"/>
@@ -6878,6 +6878,72 @@
         </is>
       </c>
       <c r="G31" s="7" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>LinkedIn Inbound (bridge)</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Channel / §3.6.6</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Inbound LinkedIn DM/InMail via extension/session (no official API)</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>POST /api/ingest/linkedin (secret) + GET/POST /api/linkedin/outbox for extension</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>PLUG extension / session</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired (server side)</t>
+        </is>
+      </c>
+      <c r="G32" s="7" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Cold Email Templates</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Outreach / §3.6.6</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>4-step cold-email sequence (subject+body, merge fields)</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>lib/templates/email-catalog + POST /api/outreach/cold-email (HITL)</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>n/a (internal)</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
docs(sdr): §3.6.7 custom/BYO templates upload
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCTS/HELIX-external-connections.xlsx
+++ b/PRODUCTS/HELIX-external-connections.xlsx
@@ -5866,7 +5866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6944,6 +6944,39 @@
         </is>
       </c>
       <c r="G33" s="7" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Custom Templates (BYO)</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Templates / §3.6.7</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Upload your own WhatsApp/email templates; override built-ins by key</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>custom_templates table + POST/GET/DELETE /api/templates/custom (single+bulk)</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>n/a (internal)</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G34" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
docs(sdr): templates management UI (/templates)
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCTS/HELIX-external-connections.xlsx
+++ b/PRODUCTS/HELIX-external-connections.xlsx
@@ -5866,7 +5866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6977,6 +6977,39 @@
         </is>
       </c>
       <c r="G34" s="7" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Templates UI</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>UI / §3.6.7</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Manage templates: view built-in + upload/edit/delete custom (WhatsApp/email/canned)</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>/templates page + /api/templates/list + /api/canned</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>n/a (internal)</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
docs(connections): reflect WhatsApp inbound bot + number linking
Update HELIX-external-connections: Rank/SEO-GEO WhatsApp 🔧→✅ (sheet + Master
+ matrix), enrich WhatsApp purpose for Dashboards/OPS/SDR/Growth-Doctor to note
the inbound bot + number linking, and add the missing HELIX Growth Doctor
column to the Channels matrix.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCTS/HELIX-external-connections.xlsx
+++ b/PRODUCTS/HELIX-external-connections.xlsx
@@ -659,7 +659,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Status: ✅ Wired = live in code  ·  🔧 Planned/Partial = in spec, not fully wired  ·  ⚪ Optional/BYO</t>
+          <t>Status: ✅ Wired = live in code  ·  🔧 Planned/Partial = in spec, not fully wired  ·  ⚪ Optional/BYO  |  Update 04.08.2026: WhatsApp inbound bot + number→account linking wired across Dashboards/Growth-Doctor/SDR/OPS/Rank; Rank WhatsApp 🔧→✅.</t>
         </is>
       </c>
     </row>
@@ -852,7 +852,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Inbound lead auto-reply + outbound + HITL approve buttons</t>
+          <t>Inbound lead auto-reply + outbound + HITL; operator number linking via /api/bot/link</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -1490,7 +1490,7 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Outbound WhatsApp (24h window / template)</t>
+          <t>Outbound (24h/template) + INBOUND operator bot via /api/webhooks/meta — number linked via bot_links</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>Bot delivery (shared engine)</t>
+          <t>Inbound operator bot (/api/whatsapp) + digest delivery — number linked to a site via channel_bindings</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
@@ -2473,7 +2473,7 @@
       </c>
       <c r="F62" s="8" t="inlineStr">
         <is>
-          <t>🔧 Partial</t>
+          <t>✅ Wired</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr"/>
@@ -3910,7 +3910,7 @@
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>Digest delivery via WhatsApp</t>
+          <t>Digest delivery (with chart image) + INBOUND bot + number linking via bot_links</t>
         </is>
       </c>
       <c r="D111" s="5" t="inlineStr">
@@ -4284,7 +4284,7 @@
       </c>
       <c r="C124" s="5" t="inlineStr">
         <is>
-          <t>Doctor digest + inbound actions</t>
+          <t>Doctor digest + INBOUND bot (/api/whatsapp) + number linking via bot_links</t>
         </is>
       </c>
       <c r="D124" s="5" t="inlineStr">
@@ -5637,7 +5637,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Doctor digest + inbound actions</t>
+          <t>Doctor digest + INBOUND bot (/api/whatsapp) + number linking via bot_links</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -6067,7 +6067,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Inbound lead auto-reply + outbound + HITL approve buttons</t>
+          <t>Inbound lead auto-reply + outbound + HITL; operator number linking via /api/bot/link</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -7231,7 +7231,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Outbound WhatsApp (24h window / template)</t>
+          <t>Outbound (24h window/template) + INBOUND operator bot via /api/webhooks/meta (messages field) — number linked via bot_links</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -8510,12 +8510,12 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Bot delivery (shared engine)</t>
+          <t>Inbound operator bot (/api/whatsapp) + digest delivery — number linked to a site via channel_bindings</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Meta app + access_token + phone_number_id</t>
+          <t>Meta app + access_token + phone_number_id + WHATSAPP_VERIFY_TOKEN</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -8525,7 +8525,7 @@
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>🔧 Partial</t>
+          <t>✅ Wired</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr"/>
@@ -10055,7 +10055,7 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Digest delivery via WhatsApp</t>
+          <t>Digest delivery (with chart image) + INBOUND bot (/api/whatsapp) + number linking via bot_links</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
@@ -10370,7 +10370,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -10418,6 +10418,11 @@
           <t>HELIX Dashboards</t>
         </is>
       </c>
+      <c r="H1" s="17" t="inlineStr">
+        <is>
+          <t>HELIX Growth Doctor</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="18" t="inlineStr">
@@ -10437,7 +10442,7 @@
       </c>
       <c r="D2" s="20" t="inlineStr">
         <is>
-          <t>🔧</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="E2" s="21" t="inlineStr"/>
@@ -10447,6 +10452,11 @@
           <t>✅</t>
         </is>
       </c>
+      <c r="H2" s="19" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="18" t="inlineStr">
@@ -10476,6 +10486,11 @@
         </is>
       </c>
       <c r="G3" s="19" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H3" s="19" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -10501,6 +10516,7 @@
       <c r="E4" s="21" t="inlineStr"/>
       <c r="F4" s="21" t="inlineStr"/>
       <c r="G4" s="21" t="inlineStr"/>
+      <c r="H4" s="21" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="18" t="inlineStr">
@@ -10522,6 +10538,7 @@
       <c r="E5" s="21" t="inlineStr"/>
       <c r="F5" s="21" t="inlineStr"/>
       <c r="G5" s="21" t="inlineStr"/>
+      <c r="H5" s="21" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="18" t="inlineStr">
@@ -10543,6 +10560,7 @@
       <c r="E6" s="21" t="inlineStr"/>
       <c r="F6" s="21" t="inlineStr"/>
       <c r="G6" s="21" t="inlineStr"/>
+      <c r="H6" s="21" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="18" t="inlineStr">
@@ -10576,6 +10594,11 @@
         </is>
       </c>
       <c r="G7" s="19" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H7" s="19" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -10597,6 +10620,7 @@
       <c r="E8" s="21" t="inlineStr"/>
       <c r="F8" s="21" t="inlineStr"/>
       <c r="G8" s="21" t="inlineStr"/>
+      <c r="H8" s="21" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="18" t="inlineStr">
@@ -10614,6 +10638,7 @@
       <c r="E9" s="21" t="inlineStr"/>
       <c r="F9" s="21" t="inlineStr"/>
       <c r="G9" s="21" t="inlineStr"/>
+      <c r="H9" s="21" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="18" t="inlineStr">
@@ -10631,6 +10656,7 @@
       <c r="E10" s="21" t="inlineStr"/>
       <c r="F10" s="21" t="inlineStr"/>
       <c r="G10" s="21" t="inlineStr"/>
+      <c r="H10" s="21" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="18" t="inlineStr">
@@ -10648,6 +10674,7 @@
       <c r="E11" s="21" t="inlineStr"/>
       <c r="F11" s="21" t="inlineStr"/>
       <c r="G11" s="21" t="inlineStr"/>
+      <c r="H11" s="21" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="18" t="inlineStr">
@@ -10669,6 +10696,11 @@
       <c r="E12" s="21" t="inlineStr"/>
       <c r="F12" s="21" t="inlineStr"/>
       <c r="G12" s="19" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H12" s="19" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
docs(ops): document performance round-2 (effective-ads parity) across product page, spec, xlsx, status doc
- app/products/products-data.ts: marketing-ops gets campaign-from-scratch, Bayesian scoring, one-click OAuth connect, white-label report & style-agent cards + narrative; TikTok Ads / Outbrain added to constellation.
- PRODUCTS/01-marketing-ops-hub.md: new round-2 subsection in 2.12; xlsx TODO closed.
- PRODUCTS/HELIX-external-connections.xlsx (HELIX OPS sheet): Meta/Google/Outbrain rows updated + new TikTok Ads mgmt, OAuth Connect, White-Label Report, Performance module rows.
- PRODUCTS/HELIX-OPS-PERFORMANCE-STATUS.docx: new what-was-done / what-to-finish doc.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCTS/HELIX-external-connections.xlsx
+++ b/PRODUCTS/HELIX-external-connections.xlsx
@@ -5967,7 +5967,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -6352,6 +6352,138 @@
         </is>
       </c>
       <c r="G13" s="24" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="24" t="inlineStr">
+        <is>
+          <t>Marketing site - 'האיזור האישי' button</t>
+        </is>
+      </c>
+      <c r="B14" s="24" t="inlineStr">
+        <is>
+          <t>Entry point</t>
+        </is>
+      </c>
+      <c r="C14" s="24" t="inlineStr">
+        <is>
+          <t>Header link (desktop+mobile) to the portal</t>
+        </is>
+      </c>
+      <c r="D14" s="24" t="inlineStr">
+        <is>
+          <t>Nav.tsx + globals.css</t>
+        </is>
+      </c>
+      <c r="E14" s="24" t="inlineStr">
+        <is>
+          <t>internal (deployed to Vercel)</t>
+        </is>
+      </c>
+      <c r="F14" s="24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G14" s="24" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="24" t="inlineStr">
+        <is>
+          <t>AccountMenu (per product app)</t>
+        </is>
+      </c>
+      <c r="B15" s="24" t="inlineStr">
+        <is>
+          <t>Entry point</t>
+        </is>
+      </c>
+      <c r="C15" s="24" t="inlineStr">
+        <is>
+          <t>Avatar menu in each product nav -&gt; portal</t>
+        </is>
+      </c>
+      <c r="D15" s="24" t="inlineStr">
+        <is>
+          <t>Paste AccountMenu.tsx into each app's nav</t>
+        </is>
+      </c>
+      <c r="E15" s="24" t="inlineStr">
+        <is>
+          <t>PRODUCTS/account-portal-handoff/AccountMenu.tsx</t>
+        </is>
+      </c>
+      <c r="F15" s="24" t="inlineStr">
+        <is>
+          <t>Ready - embed x8</t>
+        </is>
+      </c>
+      <c r="G15" s="24" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="24" t="inlineStr">
+        <is>
+          <t>Shared session cookie (.helix.co.il)</t>
+        </is>
+      </c>
+      <c r="B16" s="24" t="inlineStr">
+        <is>
+          <t>Auth / SSO</t>
+        </is>
+      </c>
+      <c r="C16" s="24" t="inlineStr">
+        <is>
+          <t>One login valid across all product subdomains</t>
+        </is>
+      </c>
+      <c r="D16" s="24" t="inlineStr">
+        <is>
+          <t>cookieOptions.domain='.helix.co.il' (prod) in every Supabase client</t>
+        </is>
+      </c>
+      <c r="E16" s="24" t="inlineStr">
+        <is>
+          <t>PRODUCTS/account-portal-handoff/SSO-shared-cookie.md</t>
+        </is>
+      </c>
+      <c r="F16" s="24" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="G16" s="24" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="24" t="inlineStr">
+        <is>
+          <t>Subdomains DNS (*.helix.co.il)</t>
+        </is>
+      </c>
+      <c r="B17" s="24" t="inlineStr">
+        <is>
+          <t>Infra / DNS</t>
+        </is>
+      </c>
+      <c r="C17" s="24" t="inlineStr">
+        <is>
+          <t>my/dashboards/sdr... on same root domain (required for SSO)</t>
+        </is>
+      </c>
+      <c r="D17" s="24" t="inlineStr">
+        <is>
+          <t>DNS records + add domains in Vercel</t>
+        </is>
+      </c>
+      <c r="E17" s="24" t="inlineStr">
+        <is>
+          <t>domain registrar + vercel.com</t>
+        </is>
+      </c>
+      <c r="F17" s="24" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="G17" s="24" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7592,7 +7724,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8321,12 +8453,12 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Full paid campaign automation (Campaign→AdSet+budget+targeting→Ads A/B) + audience segmentation + budget optimizer + per-variant insights</t>
+          <t>Full paid campaign automation (Campaign→AdSet→Ads A/B) + NEW createCampaign connector + one-click OAuth connect + budget optimizer + per-variant insights</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>FB_ADS_TOKEN + FB_AD_ACCOUNT_ID + FB_PAGE_ID (or per-workspace channel_connections 'פייסבוק')</t>
+          <t>FB_ADS_TOKEN + FB_AD_ACCOUNT_ID + FB_PAGE_ID (or channel_connections) — OAuth: META_APP_ID + META_APP_SECRET</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -8341,7 +8473,7 @@
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>needs creds</t>
+          <t>needs creds; OAuth needs App Review</t>
         </is>
       </c>
     </row>
@@ -8761,12 +8893,12 @@
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Budget / pause connector</t>
+          <t>Budget / pause + NEW createCampaign (campaignBudget+campaign, PAUSED) + one-click OAuth connect</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>GOOGLE_ADS_ACCESS_TOKEN + DEVELOPER_TOKEN + customer_id</t>
+          <t>GOOGLE_ADS_ACCESS_TOKEN + DEVELOPER_TOKEN + customer_id — OAuth: GOOGLE_OAUTH_CLIENT_ID + _SECRET</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -8776,7 +8908,12 @@
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>✅ Wired</t>
+          <t>🔧 Code ready</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>OAuth gives token; dev_token+customer_id still manual; untested live</t>
         </is>
       </c>
     </row>
@@ -8793,7 +8930,7 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Ads connector</t>
+          <t>Ads connector (pause/budget/upload) + NEW createCampaign (monthly budget, disabled)</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
@@ -8808,7 +8945,12 @@
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>✅ Wired</t>
+          <t>🔧 Code ready</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>manual token (no OAuth); untested live</t>
         </is>
       </c>
     </row>
@@ -8841,6 +8983,154 @@
       <c r="F38" s="6" t="inlineStr">
         <is>
           <t>✅ Wired</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>TikTok Ads (Ads mgmt)</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>Ads mgmt</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>Pause/budget/insights + NEW createCampaign (campaign shell, paused) + one-click OAuth connect</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>TIKTOK_ACCESS_TOKEN + TIKTOK_ADVERTISER_ID (or OAuth: TIKTOK_APP_ID + TIKTOK_APP_SECRET)</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>business-api.tiktok.com</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>🔧 Code ready</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>untested live; adgroups/ads still manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>OAuth Connect (Meta/Google/TikTok)</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Ads / Auth</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>One-click account connect (OAuth) for ad platforms → writes channel_connections.config. /api/oauth/[platform]/start+callback</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>META_APP_ID/SECRET, GOOGLE_OAUTH_CLIENT_ID/SECRET, TIKTOK_APP_ID/SECRET</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>each platform dev portal (App Review required)</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>🔧 Code ready</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>needs approved apps; falls back to manual paste</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>White-Label Report (public link)</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>Branded client performance report + public /report/[token] print-to-PDF (branding: logo/color/footer)</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>report_token (workspaces) + SUPABASE_SERVICE_ROLE_KEY (already set)</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>needs v20 SQL</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Performance module (scoring/builder/style/notify)</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Ads / AI</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>Bayesian creative scoring + AI campaign builder + style-learning agent + WhatsApp activity digest</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>ANTHROPIC_API_KEY + performance_settings/style tables + WhatsApp channel (notify)</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t>✅ Code</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>needs v19+v20 SQL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: HELIX Guard on readiness landing + @helix/prompts kit + product docs
- app/startups/readiness: Guard as GET item #07, unlocked post-connection to STAGE
- lib/prompt-kit.ts: shared structured-prompt scaffold (@helix/prompts convention,
  ported from PromptForge: role→inputs→workflow→constraints→output-contract)
- lib/content-tool.ts: all 3 prompts refactored onto prompt-kit (JSON contracts unchanged)
- PRODUCTS: 09-helix-guard (new product spec), PROMPTFORGE-ANALYSIS (new),
  04-seo-agent §13.6 act-engine built, external-connections xlsx act-loop row

typecheck green.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCTS/HELIX-external-connections.xlsx
+++ b/PRODUCTS/HELIX-external-connections.xlsx
@@ -676,7 +676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G138"/>
+  <dimension ref="A1:G140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2584,172 +2584,173 @@
       <c r="G64" s="7" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="5" t="inlineStr">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>OpenSEO (self-host)</t>
+        </is>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>Scrape / Audit</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>Optional local crawl/audit engine — act-loop uses existing Firecrawl/BrightData instead</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>Docker container</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t>github.com/.../openseo</t>
+        </is>
+      </c>
+      <c r="F65" s="4" t="inlineStr">
+        <is>
+          <t>⬜ Candidate (seo-god) — not needed; act-loop built on GSC</t>
+        </is>
+      </c>
+      <c r="G65" s="4" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>Act loop (Vercel Cron)</t>
+        </is>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>Infra / autonomy</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>Daily agent: /api/act — regressions→quick-wins 4–15→readout (built 2026-08-07)</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>ACT_SECRET env + Vercel Cron</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t>vercel.com</t>
+        </is>
+      </c>
+      <c r="F66" s="4" t="inlineStr">
+        <is>
+          <t>🟢 Built (helix-rank) — needs cron wiring + GSC token</t>
+        </is>
+      </c>
+      <c r="G66" s="4" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
         <is>
           <t>Vercel</t>
         </is>
       </c>
-      <c r="B65" s="5" t="inlineStr">
+      <c r="B67" s="5" t="inlineStr">
         <is>
           <t>Infra</t>
         </is>
       </c>
-      <c r="C65" s="5" t="inlineStr">
+      <c r="C67" s="5" t="inlineStr">
         <is>
           <t>Hosting + Cron</t>
         </is>
       </c>
-      <c r="D65" s="5" t="inlineStr">
+      <c r="D67" s="5" t="inlineStr">
         <is>
           <t>git push origin (HELIX-SEO-AND-GEO-BOT)</t>
         </is>
       </c>
-      <c r="E65" s="5" t="inlineStr">
+      <c r="E67" s="5" t="inlineStr">
         <is>
           <t>vercel.com</t>
         </is>
       </c>
-      <c r="F65" s="6" t="inlineStr">
+      <c r="F67" s="6" t="inlineStr">
         <is>
           <t>✅ Core</t>
         </is>
       </c>
-      <c r="G65" s="7" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="13" t="inlineStr">
+      <c r="G67" s="7" t="inlineStr"/>
+    </row>
+    <row r="68"/>
+    <row r="69">
+      <c r="A69" s="13" t="inlineStr">
         <is>
           <t>GEO Landing Page</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="4" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr">
         <is>
           <t>Service / Channel</t>
         </is>
       </c>
-      <c r="B68" s="4" t="inlineStr">
+      <c r="B70" s="4" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C68" s="4" t="inlineStr">
+      <c r="C70" s="4" t="inlineStr">
         <is>
           <t>Purpose</t>
         </is>
       </c>
-      <c r="D68" s="4" t="inlineStr">
+      <c r="D70" s="4" t="inlineStr">
         <is>
           <t>Connect (token / OAuth / webhook / env)</t>
         </is>
       </c>
-      <c r="E68" s="4" t="inlineStr">
+      <c r="E70" s="4" t="inlineStr">
         <is>
           <t>Where to get it</t>
         </is>
       </c>
-      <c r="F68" s="4" t="inlineStr">
+      <c r="F70" s="4" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G68" s="4" t="inlineStr">
+      <c r="G70" s="4" t="inlineStr">
         <is>
           <t>Connected?</t>
         </is>
       </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="5" t="inlineStr">
-        <is>
-          <t>Firecrawl</t>
-        </is>
-      </c>
-      <c r="B69" s="5" t="inlineStr">
-        <is>
-          <t>Scrape</t>
-        </is>
-      </c>
-      <c r="C69" s="5" t="inlineStr">
-        <is>
-          <t>Scrape/render the scanned page (JS)</t>
-        </is>
-      </c>
-      <c r="D69" s="5" t="inlineStr">
-        <is>
-          <t>FIRECRAWL_API_KEY (+ FIRECRAWL_BASE_URL)</t>
-        </is>
-      </c>
-      <c r="E69" s="5" t="inlineStr">
-        <is>
-          <t>firecrawl.dev</t>
-        </is>
-      </c>
-      <c r="F69" s="6" t="inlineStr">
-        <is>
-          <t>✅ Wired</t>
-        </is>
-      </c>
-      <c r="G69" s="7" t="inlineStr"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="5" t="inlineStr">
-        <is>
-          <t>Anthropic Claude</t>
-        </is>
-      </c>
-      <c r="B70" s="5" t="inlineStr">
-        <is>
-          <t>AI / answer-engine</t>
-        </is>
-      </c>
-      <c r="C70" s="5" t="inlineStr">
-        <is>
-          <t>AI-visibility scoring</t>
-        </is>
-      </c>
-      <c r="D70" s="5" t="inlineStr">
-        <is>
-          <t>ANTHROPIC_API_KEY</t>
-        </is>
-      </c>
-      <c r="E70" s="5" t="inlineStr">
-        <is>
-          <t>console.anthropic.com</t>
-        </is>
-      </c>
-      <c r="F70" s="6" t="inlineStr">
-        <is>
-          <t>✅ Wired</t>
-        </is>
-      </c>
-      <c r="G70" s="7" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>OpenAI (ChatGPT)</t>
+          <t>Firecrawl</t>
         </is>
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>AI / answer-engine</t>
+          <t>Scrape</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>AI-visibility scoring across engines</t>
+          <t>Scrape/render the scanned page (JS)</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>OPENAI_API_KEY</t>
+          <t>FIRECRAWL_API_KEY (+ FIRECRAWL_BASE_URL)</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t>platform.openai.com</t>
+          <t>firecrawl.dev</t>
         </is>
       </c>
       <c r="F71" s="6" t="inlineStr">
@@ -2762,7 +2763,7 @@
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>Google Gemini</t>
+          <t>Anthropic Claude</t>
         </is>
       </c>
       <c r="B72" s="5" t="inlineStr">
@@ -2772,17 +2773,17 @@
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>AI-visibility check (Gemini/AI Overviews)</t>
+          <t>AI-visibility scoring</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>GEMINI_API_KEY</t>
+          <t>ANTHROPIC_API_KEY</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t>aistudio.google.com</t>
+          <t>console.anthropic.com</t>
         </is>
       </c>
       <c r="F72" s="6" t="inlineStr">
@@ -2795,7 +2796,7 @@
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>Perplexity</t>
+          <t>OpenAI (ChatGPT)</t>
         </is>
       </c>
       <c r="B73" s="5" t="inlineStr">
@@ -2805,17 +2806,17 @@
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>AI-visibility check (Perplexity)</t>
+          <t>AI-visibility scoring across engines</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>PERPLEXITY_API_KEY</t>
+          <t>OPENAI_API_KEY</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t>perplexity.ai/settings/api</t>
+          <t>platform.openai.com</t>
         </is>
       </c>
       <c r="F73" s="6" t="inlineStr">
@@ -2828,32 +2829,32 @@
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>DataForSEO</t>
+          <t>Google Gemini</t>
         </is>
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>SEO data</t>
+          <t>AI / answer-engine</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>SERP / keyword / ranking data</t>
+          <t>AI-visibility check (Gemini/AI Overviews)</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>DATAFORSEO_LOGIN / DATAFORSEO_PASSWORD</t>
+          <t>GEMINI_API_KEY</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
         <is>
-          <t>dataforseo.com</t>
+          <t>aistudio.google.com</t>
         </is>
       </c>
       <c r="F74" s="6" t="inlineStr">
         <is>
-          <t>⬜ Not in code (other app)</t>
+          <t>✅ Wired</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr"/>
@@ -2861,32 +2862,32 @@
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>Serper</t>
+          <t>Perplexity</t>
         </is>
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>SEO data</t>
+          <t>AI / answer-engine</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Google SERP results API</t>
+          <t>AI-visibility check (Perplexity)</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>SERPER_API_KEY</t>
+          <t>PERPLEXITY_API_KEY</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t>serper.dev</t>
+          <t>perplexity.ai/settings/api</t>
         </is>
       </c>
       <c r="F75" s="6" t="inlineStr">
         <is>
-          <t>⬜ Not in code (other app)</t>
+          <t>✅ Wired</t>
         </is>
       </c>
       <c r="G75" s="7" t="inlineStr"/>
@@ -2894,7 +2895,7 @@
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>Google Search Console</t>
+          <t>DataForSEO</t>
         </is>
       </c>
       <c r="B76" s="5" t="inlineStr">
@@ -2904,17 +2905,17 @@
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>Rankings/impressions (OAuth)</t>
+          <t>SERP / keyword / ranking data</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>GOOGLE_CLIENT_ID / _SECRET / _REDIRECT_URI</t>
+          <t>DATAFORSEO_LOGIN / DATAFORSEO_PASSWORD</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t>console.cloud.google.com</t>
+          <t>dataforseo.com</t>
         </is>
       </c>
       <c r="F76" s="6" t="inlineStr">
@@ -2927,32 +2928,32 @@
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>Supabase</t>
+          <t>Serper</t>
         </is>
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>Core / DB</t>
+          <t>SEO data</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Lead capture (scan → email)</t>
+          <t>Google SERP results API</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>NEXT_PUBLIC_SUPABASE_URL / _ANON_KEY / SUPABASE_SERVICE_ROLE_KEY</t>
+          <t>SERPER_API_KEY</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t>supabase.com</t>
+          <t>serper.dev</t>
         </is>
       </c>
       <c r="F77" s="6" t="inlineStr">
         <is>
-          <t>✅ Wired</t>
+          <t>⬜ Not in code (other app)</t>
         </is>
       </c>
       <c r="G77" s="7" t="inlineStr"/>
@@ -2960,32 +2961,32 @@
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
         <is>
-          <t>Email (Resend)</t>
+          <t>Google Search Console</t>
         </is>
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>Channel</t>
+          <t>SEO data</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>Notify on new lead</t>
+          <t>Rankings/impressions (OAuth)</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>RESEND_API_KEY / RESEND_NOTIFY_TO</t>
+          <t>GOOGLE_CLIENT_ID / _SECRET / _REDIRECT_URI</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t>resend.com</t>
+          <t>console.cloud.google.com</t>
         </is>
       </c>
       <c r="F78" s="6" t="inlineStr">
         <is>
-          <t>✅ Wired</t>
+          <t>⬜ Not in code (other app)</t>
         </is>
       </c>
       <c r="G78" s="7" t="inlineStr"/>
@@ -2993,27 +2994,27 @@
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>WhatsApp click-to-chat</t>
+          <t>Supabase</t>
         </is>
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>Channel</t>
+          <t>Core / DB</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Contact button (wa.me link — no API)</t>
+          <t>Lead capture (scan → email)</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>wa.me link (no key)</t>
+          <t>NEXT_PUBLIC_SUPABASE_URL / _ANON_KEY / SUPABASE_SERVICE_ROLE_KEY</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>supabase.com</t>
         </is>
       </c>
       <c r="F79" s="6" t="inlineStr">
@@ -3026,27 +3027,27 @@
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
         <is>
-          <t>Google Analytics (GA)</t>
+          <t>Email (Resend)</t>
         </is>
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>Tracking</t>
+          <t>Channel</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>Site analytics</t>
+          <t>Notify on new lead</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>NEXT_PUBLIC_GA_ID</t>
+          <t>RESEND_API_KEY / RESEND_NOTIFY_TO</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t>analytics.google.com</t>
+          <t>resend.com</t>
         </is>
       </c>
       <c r="F80" s="6" t="inlineStr">
@@ -3059,27 +3060,27 @@
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>Facebook Pixel</t>
+          <t>WhatsApp click-to-chat</t>
         </is>
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>Tracking</t>
+          <t>Channel</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Ad conversion tracking</t>
+          <t>Contact button (wa.me link — no API)</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>NEXT_PUBLIC_FB_PIXEL_ID</t>
+          <t>wa.me link (no key)</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t>business.facebook.com</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F81" s="6" t="inlineStr">
@@ -3092,32 +3093,32 @@
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>Make.com</t>
+          <t>Google Analytics (GA)</t>
         </is>
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>Automation</t>
+          <t>Tracking</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>Route leads / trigger flows (webhook)</t>
+          <t>Site analytics</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>MAKE_WEBHOOK_URL</t>
+          <t>NEXT_PUBLIC_GA_ID</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t>make.com</t>
-        </is>
-      </c>
-      <c r="F82" s="11" t="inlineStr">
-        <is>
-          <t>⚪ Optional</t>
+          <t>analytics.google.com</t>
+        </is>
+      </c>
+      <c r="F82" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
         </is>
       </c>
       <c r="G82" s="7" t="inlineStr"/>
@@ -3125,32 +3126,32 @@
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>n8n</t>
+          <t>Facebook Pixel</t>
         </is>
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>Automation</t>
+          <t>Tracking</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Route leads / automation (webhook)</t>
+          <t>Ad conversion tracking</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>N8N_WEBHOOK_URL</t>
+          <t>NEXT_PUBLIC_FB_PIXEL_ID</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t>self-host n8n</t>
-        </is>
-      </c>
-      <c r="F83" s="11" t="inlineStr">
-        <is>
-          <t>⚪ Optional</t>
+          <t>business.facebook.com</t>
+        </is>
+      </c>
+      <c r="F83" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
         </is>
       </c>
       <c r="G83" s="7" t="inlineStr"/>
@@ -3158,32 +3159,32 @@
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>Dicebear</t>
+          <t>Make.com</t>
         </is>
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>Assets (free)</t>
+          <t>Automation</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>Generated avatars</t>
+          <t>Route leads / trigger flows (webhook)</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>no key (public API)</t>
+          <t>MAKE_WEBHOOK_URL</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
         <is>
-          <t>dicebear.com</t>
-        </is>
-      </c>
-      <c r="F84" s="6" t="inlineStr">
-        <is>
-          <t>⬜ Not in code (other app)</t>
+          <t>make.com</t>
+        </is>
+      </c>
+      <c r="F84" s="11" t="inlineStr">
+        <is>
+          <t>⚪ Optional</t>
         </is>
       </c>
       <c r="G84" s="7" t="inlineStr"/>
@@ -3191,27 +3192,27 @@
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>ipapi.co</t>
+          <t>n8n</t>
         </is>
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>Data (free)</t>
+          <t>Automation</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Visitor geo-IP</t>
+          <t>Route leads / automation (webhook)</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>no key (free tier)</t>
+          <t>N8N_WEBHOOK_URL</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
         <is>
-          <t>ipapi.co</t>
+          <t>self-host n8n</t>
         </is>
       </c>
       <c r="F85" s="11" t="inlineStr">
@@ -3224,17 +3225,17 @@
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>CommonCrawl</t>
+          <t>Dicebear</t>
         </is>
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>Data (free)</t>
+          <t>Assets (free)</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>Is the page in the crawl index</t>
+          <t>Generated avatars</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
@@ -3244,12 +3245,12 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t>index.commoncrawl.org</t>
+          <t>dicebear.com</t>
         </is>
       </c>
       <c r="F86" s="6" t="inlineStr">
         <is>
-          <t>✅ Wired</t>
+          <t>⬜ Not in code (other app)</t>
         </is>
       </c>
       <c r="G86" s="7" t="inlineStr"/>
@@ -3257,7 +3258,7 @@
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>Wikidata</t>
+          <t>ipapi.co</t>
         </is>
       </c>
       <c r="B87" s="5" t="inlineStr">
@@ -3267,22 +3268,22 @@
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Entity / knowledge-graph presence</t>
+          <t>Visitor geo-IP</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>no key (public API)</t>
+          <t>no key (free tier)</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t>wikidata.org</t>
-        </is>
-      </c>
-      <c r="F87" s="6" t="inlineStr">
-        <is>
-          <t>✅ Wired</t>
+          <t>ipapi.co</t>
+        </is>
+      </c>
+      <c r="F87" s="11" t="inlineStr">
+        <is>
+          <t>⚪ Optional</t>
         </is>
       </c>
       <c r="G87" s="7" t="inlineStr"/>
@@ -3290,32 +3291,32 @@
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>Webhook / API secrets</t>
+          <t>CommonCrawl</t>
         </is>
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>Infra</t>
+          <t>Data (free)</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>Protect inbound webhooks</t>
+          <t>Is the page in the crawl index</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>WEBHOOK_SECRET / API_KEY</t>
+          <t>no key (public API)</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t>self-chosen</t>
+          <t>index.commoncrawl.org</t>
         </is>
       </c>
       <c r="F88" s="6" t="inlineStr">
         <is>
-          <t>⬜ Not in code (IP rate-limit + honeypot only)</t>
+          <t>✅ Wired</t>
         </is>
       </c>
       <c r="G88" s="7" t="inlineStr"/>
@@ -3323,175 +3324,176 @@
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
+          <t>Wikidata</t>
+        </is>
+      </c>
+      <c r="B89" s="5" t="inlineStr">
+        <is>
+          <t>Data (free)</t>
+        </is>
+      </c>
+      <c r="C89" s="5" t="inlineStr">
+        <is>
+          <t>Entity / knowledge-graph presence</t>
+        </is>
+      </c>
+      <c r="D89" s="5" t="inlineStr">
+        <is>
+          <t>no key (public API)</t>
+        </is>
+      </c>
+      <c r="E89" s="5" t="inlineStr">
+        <is>
+          <t>wikidata.org</t>
+        </is>
+      </c>
+      <c r="F89" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G89" s="7" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="5" t="inlineStr">
+        <is>
+          <t>Webhook / API secrets</t>
+        </is>
+      </c>
+      <c r="B90" s="5" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="C90" s="5" t="inlineStr">
+        <is>
+          <t>Protect inbound webhooks</t>
+        </is>
+      </c>
+      <c r="D90" s="5" t="inlineStr">
+        <is>
+          <t>WEBHOOK_SECRET / API_KEY</t>
+        </is>
+      </c>
+      <c r="E90" s="5" t="inlineStr">
+        <is>
+          <t>self-chosen</t>
+        </is>
+      </c>
+      <c r="F90" s="6" t="inlineStr">
+        <is>
+          <t>⬜ Not in code (IP rate-limit + honeypot only)</t>
+        </is>
+      </c>
+      <c r="G90" s="7" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="5" t="inlineStr">
+        <is>
           <t>Vercel</t>
         </is>
       </c>
-      <c r="B89" s="5" t="inlineStr">
+      <c r="B91" s="5" t="inlineStr">
         <is>
           <t>Infra</t>
         </is>
       </c>
-      <c r="C89" s="5" t="inlineStr">
+      <c r="C91" s="5" t="inlineStr">
         <is>
           <t>Hosting (helix website repo)</t>
         </is>
       </c>
-      <c r="D89" s="5" t="inlineStr">
+      <c r="D91" s="5" t="inlineStr">
         <is>
           <t>git push vercel master</t>
         </is>
       </c>
-      <c r="E89" s="5" t="inlineStr">
+      <c r="E91" s="5" t="inlineStr">
         <is>
           <t>vercel.com</t>
         </is>
       </c>
-      <c r="F89" s="6" t="inlineStr">
+      <c r="F91" s="6" t="inlineStr">
         <is>
           <t>✅ Core</t>
         </is>
       </c>
-      <c r="G89" s="7" t="inlineStr"/>
-    </row>
-    <row r="91">
-      <c r="A91" s="14" t="inlineStr">
+      <c r="G91" s="7" t="inlineStr"/>
+    </row>
+    <row r="92"/>
+    <row r="93">
+      <c r="A93" s="14" t="inlineStr">
         <is>
           <t>HELIX STAGE</t>
         </is>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" s="4" t="inlineStr">
+    <row r="94">
+      <c r="A94" s="4" t="inlineStr">
         <is>
           <t>Service / Channel</t>
         </is>
       </c>
-      <c r="B92" s="4" t="inlineStr">
+      <c r="B94" s="4" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C92" s="4" t="inlineStr">
+      <c r="C94" s="4" t="inlineStr">
         <is>
           <t>Purpose</t>
         </is>
       </c>
-      <c r="D92" s="4" t="inlineStr">
+      <c r="D94" s="4" t="inlineStr">
         <is>
           <t>Connect (token / OAuth / webhook / env)</t>
         </is>
       </c>
-      <c r="E92" s="4" t="inlineStr">
+      <c r="E94" s="4" t="inlineStr">
         <is>
           <t>Where to get it</t>
         </is>
       </c>
-      <c r="F92" s="4" t="inlineStr">
+      <c r="F94" s="4" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G92" s="4" t="inlineStr">
+      <c r="G94" s="4" t="inlineStr">
         <is>
           <t>Connected?</t>
         </is>
       </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="5" t="inlineStr">
-        <is>
-          <t>Supabase</t>
-        </is>
-      </c>
-      <c r="B93" s="5" t="inlineStr">
-        <is>
-          <t>Core / DB</t>
-        </is>
-      </c>
-      <c r="C93" s="5" t="inlineStr">
-        <is>
-          <t>Launches, votes, comments, products + Auth</t>
-        </is>
-      </c>
-      <c r="D93" s="5" t="inlineStr">
-        <is>
-          <t>NEXT_PUBLIC_SUPABASE_URL / _ANON_KEY / SERVICE_ROLE</t>
-        </is>
-      </c>
-      <c r="E93" s="5" t="inlineStr">
-        <is>
-          <t>supabase.com</t>
-        </is>
-      </c>
-      <c r="F93" s="6" t="inlineStr">
-        <is>
-          <t>✅ Wired</t>
-        </is>
-      </c>
-      <c r="G93" s="7" t="inlineStr"/>
-    </row>
-    <row r="94">
-      <c r="A94" s="5" t="inlineStr">
-        <is>
-          <t>Email (Resend)</t>
-        </is>
-      </c>
-      <c r="B94" s="5" t="inlineStr">
-        <is>
-          <t>Channel</t>
-        </is>
-      </c>
-      <c r="C94" s="5" t="inlineStr">
-        <is>
-          <t>Owner notifications (new comment/vote)</t>
-        </is>
-      </c>
-      <c r="D94" s="5" t="inlineStr">
-        <is>
-          <t>RESEND_API_KEY / RESEND_FROM</t>
-        </is>
-      </c>
-      <c r="E94" s="5" t="inlineStr">
-        <is>
-          <t>resend.com</t>
-        </is>
-      </c>
-      <c r="F94" s="6" t="inlineStr">
-        <is>
-          <t>✅ Wired</t>
-        </is>
-      </c>
-      <c r="G94" s="7" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
         <is>
-          <t>Telegram Bot</t>
+          <t>Supabase</t>
         </is>
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>Channel</t>
+          <t>Core / DB</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>Optional owner pings (shared bot engine)</t>
+          <t>Launches, votes, comments, products + Auth</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>bot_token + chat_id</t>
+          <t>NEXT_PUBLIC_SUPABASE_URL / _ANON_KEY / SERVICE_ROLE</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t>@BotFather</t>
-        </is>
-      </c>
-      <c r="F95" s="11" t="inlineStr">
-        <is>
-          <t>⚪ Optional</t>
+          <t>supabase.com</t>
+        </is>
+      </c>
+      <c r="F95" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
         </is>
       </c>
       <c r="G95" s="7" t="inlineStr"/>
@@ -3499,27 +3501,27 @@
     <row r="96">
       <c r="A96" s="5" t="inlineStr">
         <is>
-          <t>Cron secrets</t>
+          <t>Email (Resend)</t>
         </is>
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>Infra</t>
+          <t>Channel</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>Protect scheduled routes</t>
+          <t>Owner notifications (new comment/vote)</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>CRON_SECRET / DIGEST_SECRET</t>
+          <t>RESEND_API_KEY / RESEND_FROM</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t>self-chosen</t>
+          <t>resend.com</t>
         </is>
       </c>
       <c r="F96" s="6" t="inlineStr">
@@ -3532,170 +3534,171 @@
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
         <is>
+          <t>Telegram Bot</t>
+        </is>
+      </c>
+      <c r="B97" s="5" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="C97" s="5" t="inlineStr">
+        <is>
+          <t>Optional owner pings (shared bot engine)</t>
+        </is>
+      </c>
+      <c r="D97" s="5" t="inlineStr">
+        <is>
+          <t>bot_token + chat_id</t>
+        </is>
+      </c>
+      <c r="E97" s="5" t="inlineStr">
+        <is>
+          <t>@BotFather</t>
+        </is>
+      </c>
+      <c r="F97" s="11" t="inlineStr">
+        <is>
+          <t>⚪ Optional</t>
+        </is>
+      </c>
+      <c r="G97" s="7" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="5" t="inlineStr">
+        <is>
+          <t>Cron secrets</t>
+        </is>
+      </c>
+      <c r="B98" s="5" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="C98" s="5" t="inlineStr">
+        <is>
+          <t>Protect scheduled routes</t>
+        </is>
+      </c>
+      <c r="D98" s="5" t="inlineStr">
+        <is>
+          <t>CRON_SECRET / DIGEST_SECRET</t>
+        </is>
+      </c>
+      <c r="E98" s="5" t="inlineStr">
+        <is>
+          <t>self-chosen</t>
+        </is>
+      </c>
+      <c r="F98" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G98" s="7" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="5" t="inlineStr">
+        <is>
           <t>Vercel</t>
         </is>
       </c>
-      <c r="B97" s="5" t="inlineStr">
+      <c r="B99" s="5" t="inlineStr">
         <is>
           <t>Infra</t>
         </is>
       </c>
-      <c r="C97" s="5" t="inlineStr">
+      <c r="C99" s="5" t="inlineStr">
         <is>
           <t>Hosting + Cron</t>
         </is>
       </c>
-      <c r="D97" s="5" t="inlineStr">
+      <c r="D99" s="5" t="inlineStr">
         <is>
           <t>git push</t>
         </is>
       </c>
-      <c r="E97" s="5" t="inlineStr">
+      <c r="E99" s="5" t="inlineStr">
         <is>
           <t>vercel.com</t>
         </is>
       </c>
-      <c r="F97" s="6" t="inlineStr">
+      <c r="F99" s="6" t="inlineStr">
         <is>
           <t>✅ Core</t>
         </is>
       </c>
-      <c r="G97" s="7" t="inlineStr"/>
-    </row>
-    <row r="99">
-      <c r="A99" s="15" t="inlineStr">
+      <c r="G99" s="7" t="inlineStr"/>
+    </row>
+    <row r="100"/>
+    <row r="101">
+      <c r="A101" s="15" t="inlineStr">
         <is>
           <t>HELIX Dashboards (Product 02)</t>
         </is>
       </c>
     </row>
-    <row r="100">
-      <c r="A100" s="4" t="inlineStr">
+    <row r="102">
+      <c r="A102" s="4" t="inlineStr">
         <is>
           <t>Service / Channel</t>
         </is>
       </c>
-      <c r="B100" s="4" t="inlineStr">
+      <c r="B102" s="4" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C100" s="4" t="inlineStr">
+      <c r="C102" s="4" t="inlineStr">
         <is>
           <t>Purpose</t>
         </is>
       </c>
-      <c r="D100" s="4" t="inlineStr">
+      <c r="D102" s="4" t="inlineStr">
         <is>
           <t>Connect (token / OAuth / webhook / env)</t>
         </is>
       </c>
-      <c r="E100" s="4" t="inlineStr">
+      <c r="E102" s="4" t="inlineStr">
         <is>
           <t>Where to get it</t>
         </is>
       </c>
-      <c r="F100" s="4" t="inlineStr">
+      <c r="F102" s="4" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G100" s="4" t="inlineStr">
+      <c r="G102" s="4" t="inlineStr">
         <is>
           <t>Connected?</t>
         </is>
       </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="5" t="inlineStr">
-        <is>
-          <t>Supabase</t>
-        </is>
-      </c>
-      <c r="B101" s="5" t="inlineStr">
-        <is>
-          <t>Core / DB</t>
-        </is>
-      </c>
-      <c r="C101" s="5" t="inlineStr">
-        <is>
-          <t>Widgets, dashboards, connector tokens (encrypted) + Auth</t>
-        </is>
-      </c>
-      <c r="D101" s="5" t="inlineStr">
-        <is>
-          <t>NEXT_PUBLIC_SUPABASE_URL / _ANON_KEY / SUPABASE_SERVICE_ROLE_KEY</t>
-        </is>
-      </c>
-      <c r="E101" s="5" t="inlineStr">
-        <is>
-          <t>supabase.com</t>
-        </is>
-      </c>
-      <c r="F101" s="6" t="inlineStr">
-        <is>
-          <t>✅ Wired</t>
-        </is>
-      </c>
-      <c r="G101" s="7" t="inlineStr"/>
-    </row>
-    <row r="102">
-      <c r="A102" s="5" t="inlineStr">
-        <is>
-          <t>Anthropic Claude</t>
-        </is>
-      </c>
-      <c r="B102" s="5" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="C102" s="5" t="inlineStr">
-        <is>
-          <t>Narrate metrics + daily digest text</t>
-        </is>
-      </c>
-      <c r="D102" s="5" t="inlineStr">
-        <is>
-          <t>ANTHROPIC_API_KEY (+ CONTENT_MODEL)</t>
-        </is>
-      </c>
-      <c r="E102" s="5" t="inlineStr">
-        <is>
-          <t>console.anthropic.com</t>
-        </is>
-      </c>
-      <c r="F102" s="6" t="inlineStr">
-        <is>
-          <t>✅ Wired</t>
-        </is>
-      </c>
-      <c r="G102" s="7" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="5" t="inlineStr">
         <is>
-          <t>Ollama</t>
+          <t>Supabase</t>
         </is>
       </c>
       <c r="B103" s="5" t="inlineStr">
         <is>
-          <t>AI / local</t>
+          <t>Core / DB</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>Local narration/classify — cost lever</t>
+          <t>Widgets, dashboards, connector tokens (encrypted) + Auth</t>
         </is>
       </c>
       <c r="D103" s="5" t="inlineStr">
         <is>
-          <t>OLLAMA_BASE_URL / OLLAMA_MODEL</t>
+          <t>NEXT_PUBLIC_SUPABASE_URL / _ANON_KEY / SUPABASE_SERVICE_ROLE_KEY</t>
         </is>
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t>ollama.com</t>
+          <t>supabase.com</t>
         </is>
       </c>
       <c r="F103" s="6" t="inlineStr">
@@ -3708,27 +3711,27 @@
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>Google Analytics (GA4)</t>
+          <t>Anthropic Claude</t>
         </is>
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>Data source</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>Traffic metrics into dashboards</t>
+          <t>Narrate metrics + daily digest text</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr">
         <is>
-          <t>GOOGLE_OAUTH_CLIENT_ID / _SECRET / _REDIRECT_URI</t>
+          <t>ANTHROPIC_API_KEY (+ CONTENT_MODEL)</t>
         </is>
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t>console.cloud.google.com</t>
+          <t>console.anthropic.com</t>
         </is>
       </c>
       <c r="F104" s="6" t="inlineStr">
@@ -3741,27 +3744,27 @@
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Ollama</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>Data source</t>
+          <t>AI / local</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>Revenue / MRR metrics</t>
+          <t>Local narration/classify — cost lever</t>
         </is>
       </c>
       <c r="D105" s="5" t="inlineStr">
         <is>
-          <t>Stripe connector token (encrypted via SECRETS_KEY)</t>
+          <t>OLLAMA_BASE_URL / OLLAMA_MODEL</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t>dashboard.stripe.com/apikeys</t>
+          <t>ollama.com</t>
         </is>
       </c>
       <c r="F105" s="6" t="inlineStr">
@@ -3774,7 +3777,7 @@
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>Plausible Analytics</t>
+          <t>Google Analytics (GA4)</t>
         </is>
       </c>
       <c r="B106" s="5" t="inlineStr">
@@ -3784,17 +3787,17 @@
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>Privacy analytics metrics</t>
+          <t>Traffic metrics into dashboards</t>
         </is>
       </c>
       <c r="D106" s="5" t="inlineStr">
         <is>
-          <t>Plausible API key (connector)</t>
+          <t>GOOGLE_OAUTH_CLIENT_ID / _SECRET / _REDIRECT_URI</t>
         </is>
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t>plausible.io</t>
+          <t>console.cloud.google.com</t>
         </is>
       </c>
       <c r="F106" s="6" t="inlineStr">
@@ -3807,7 +3810,7 @@
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>Meta / Facebook Insights</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="B107" s="5" t="inlineStr">
@@ -3817,17 +3820,17 @@
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>Social page/post insights</t>
+          <t>Revenue / MRR metrics</t>
         </is>
       </c>
       <c r="D107" s="5" t="inlineStr">
         <is>
-          <t>FB_APP_ID / FB_APP_SECRET</t>
+          <t>Stripe connector token (encrypted via SECRETS_KEY)</t>
         </is>
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t>developers.facebook.com</t>
+          <t>dashboard.stripe.com/apikeys</t>
         </is>
       </c>
       <c r="F107" s="6" t="inlineStr">
@@ -3840,7 +3843,7 @@
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>Metrics ingest (from HELIX products)</t>
+          <t>Plausible Analytics</t>
         </is>
       </c>
       <c r="B108" s="5" t="inlineStr">
@@ -3850,17 +3853,17 @@
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>Receives pushed metrics (SDR/OPS/SEO-GEO → dashboards)</t>
+          <t>Privacy analytics metrics</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
         <is>
-          <t>PULL via /api/connectors/sync + /api/cron/sync (CRON_SECRET) — no HELIX_DASHBOARDS_KEY</t>
+          <t>Plausible API key (connector)</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">
         <is>
-          <t>internal</t>
+          <t>plausible.io</t>
         </is>
       </c>
       <c r="F108" s="6" t="inlineStr">
@@ -3873,27 +3876,27 @@
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>Email (Resend)</t>
+          <t>Meta / Facebook Insights</t>
         </is>
       </c>
       <c r="B109" s="5" t="inlineStr">
         <is>
-          <t>Channel</t>
+          <t>Data source</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>Deliver daily digest / reports</t>
+          <t>Social page/post insights</t>
         </is>
       </c>
       <c r="D109" s="5" t="inlineStr">
         <is>
-          <t>RESEND_API_KEY / EMAIL_FROM</t>
+          <t>FB_APP_ID / FB_APP_SECRET</t>
         </is>
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t>resend.com</t>
+          <t>developers.facebook.com</t>
         </is>
       </c>
       <c r="F109" s="6" t="inlineStr">
@@ -3906,27 +3909,27 @@
     <row r="110">
       <c r="A110" s="5" t="inlineStr">
         <is>
-          <t>Telegram Bot</t>
+          <t>Metrics ingest (from HELIX products)</t>
         </is>
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>Channel</t>
+          <t>Data source</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>Digest delivery + bot</t>
+          <t>Receives pushed metrics (SDR/OPS/SEO-GEO → dashboards)</t>
         </is>
       </c>
       <c r="D110" s="5" t="inlineStr">
         <is>
-          <t>TELEGRAM_BOT_TOKEN</t>
+          <t>PULL via /api/connectors/sync + /api/cron/sync (CRON_SECRET) — no HELIX_DASHBOARDS_KEY</t>
         </is>
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t>@BotFather</t>
+          <t>internal</t>
         </is>
       </c>
       <c r="F110" s="6" t="inlineStr">
@@ -3939,7 +3942,7 @@
     <row r="111">
       <c r="A111" s="5" t="inlineStr">
         <is>
-          <t>WhatsApp Cloud API</t>
+          <t>Email (Resend)</t>
         </is>
       </c>
       <c r="B111" s="5" t="inlineStr">
@@ -3949,17 +3952,17 @@
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>Digest delivery (with chart image) + INBOUND bot + number linking via bot_links</t>
+          <t>Deliver daily digest / reports</t>
         </is>
       </c>
       <c r="D111" s="5" t="inlineStr">
         <is>
-          <t>WHATSAPP_TOKEN / WHATSAPP_PHONE_ID</t>
+          <t>RESEND_API_KEY / EMAIL_FROM</t>
         </is>
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t>developers.facebook.com</t>
+          <t>resend.com</t>
         </is>
       </c>
       <c r="F111" s="6" t="inlineStr">
@@ -3972,27 +3975,27 @@
     <row r="112">
       <c r="A112" s="5" t="inlineStr">
         <is>
-          <t>Secrets / Cron</t>
+          <t>Telegram Bot</t>
         </is>
       </c>
       <c r="B112" s="5" t="inlineStr">
         <is>
-          <t>Infra</t>
+          <t>Channel</t>
         </is>
       </c>
       <c r="C112" s="5" t="inlineStr">
         <is>
-          <t>Encrypt connector tokens + schedule digests</t>
+          <t>Digest delivery + bot</t>
         </is>
       </c>
       <c r="D112" s="5" t="inlineStr">
         <is>
-          <t>SECRETS_KEY / CRON_SECRET</t>
+          <t>TELEGRAM_BOT_TOKEN</t>
         </is>
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t>self-chosen</t>
+          <t>@BotFather</t>
         </is>
       </c>
       <c r="F112" s="6" t="inlineStr">
@@ -4005,170 +4008,171 @@
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
+          <t>WhatsApp Cloud API</t>
+        </is>
+      </c>
+      <c r="B113" s="5" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="C113" s="5" t="inlineStr">
+        <is>
+          <t>Digest delivery (with chart image) + INBOUND bot + number linking via bot_links</t>
+        </is>
+      </c>
+      <c r="D113" s="5" t="inlineStr">
+        <is>
+          <t>WHATSAPP_TOKEN / WHATSAPP_PHONE_ID</t>
+        </is>
+      </c>
+      <c r="E113" s="5" t="inlineStr">
+        <is>
+          <t>developers.facebook.com</t>
+        </is>
+      </c>
+      <c r="F113" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G113" s="7" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="5" t="inlineStr">
+        <is>
+          <t>Secrets / Cron</t>
+        </is>
+      </c>
+      <c r="B114" s="5" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="C114" s="5" t="inlineStr">
+        <is>
+          <t>Encrypt connector tokens + schedule digests</t>
+        </is>
+      </c>
+      <c r="D114" s="5" t="inlineStr">
+        <is>
+          <t>SECRETS_KEY / CRON_SECRET</t>
+        </is>
+      </c>
+      <c r="E114" s="5" t="inlineStr">
+        <is>
+          <t>self-chosen</t>
+        </is>
+      </c>
+      <c r="F114" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G114" s="7" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="5" t="inlineStr">
+        <is>
           <t>Vercel</t>
         </is>
       </c>
-      <c r="B113" s="5" t="inlineStr">
+      <c r="B115" s="5" t="inlineStr">
         <is>
           <t>Infra</t>
         </is>
       </c>
-      <c r="C113" s="5" t="inlineStr">
+      <c r="C115" s="5" t="inlineStr">
         <is>
           <t>Hosting + Cron</t>
         </is>
       </c>
-      <c r="D113" s="5" t="inlineStr">
+      <c r="D115" s="5" t="inlineStr">
         <is>
           <t>git push (HELIX-DASHBOARDS)</t>
         </is>
       </c>
-      <c r="E113" s="5" t="inlineStr">
+      <c r="E115" s="5" t="inlineStr">
         <is>
           <t>vercel.com</t>
         </is>
       </c>
-      <c r="F113" s="6" t="inlineStr">
+      <c r="F115" s="6" t="inlineStr">
         <is>
           <t>✅ Core</t>
         </is>
       </c>
-      <c r="G113" s="7" t="inlineStr"/>
-    </row>
-    <row r="115">
-      <c r="A115" s="15" t="inlineStr">
+      <c r="G115" s="7" t="inlineStr"/>
+    </row>
+    <row r="116"/>
+    <row r="117">
+      <c r="A117" s="15" t="inlineStr">
         <is>
           <t>HELIX Growth Doctor (Product 07)</t>
         </is>
       </c>
     </row>
-    <row r="116">
-      <c r="A116" s="4" t="inlineStr">
+    <row r="118">
+      <c r="A118" s="4" t="inlineStr">
         <is>
           <t>Service / Channel</t>
         </is>
       </c>
-      <c r="B116" s="4" t="inlineStr">
+      <c r="B118" s="4" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C116" s="4" t="inlineStr">
+      <c r="C118" s="4" t="inlineStr">
         <is>
           <t>Purpose</t>
         </is>
       </c>
-      <c r="D116" s="4" t="inlineStr">
+      <c r="D118" s="4" t="inlineStr">
         <is>
           <t>Connect (token / OAuth / webhook / env)</t>
         </is>
       </c>
-      <c r="E116" s="4" t="inlineStr">
+      <c r="E118" s="4" t="inlineStr">
         <is>
           <t>Where to get it</t>
         </is>
       </c>
-      <c r="F116" s="4" t="inlineStr">
+      <c r="F118" s="4" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G116" s="4" t="inlineStr">
+      <c r="G118" s="4" t="inlineStr">
         <is>
           <t>Connected?</t>
         </is>
       </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="5" t="inlineStr">
-        <is>
-          <t>Supabase</t>
-        </is>
-      </c>
-      <c r="B117" s="5" t="inlineStr">
-        <is>
-          <t>Core / DB</t>
-        </is>
-      </c>
-      <c r="C117" s="5" t="inlineStr">
-        <is>
-          <t>Events (funnel/returns) + cohorts + insights + Auth + RLS</t>
-        </is>
-      </c>
-      <c r="D117" s="5" t="inlineStr">
-        <is>
-          <t>NEXT_PUBLIC_SUPABASE_URL / _ANON_KEY / SUPABASE_SERVICE_ROLE_KEY</t>
-        </is>
-      </c>
-      <c r="E117" s="5" t="inlineStr">
-        <is>
-          <t>supabase.com</t>
-        </is>
-      </c>
-      <c r="F117" s="6" t="inlineStr">
-        <is>
-          <t>✅ Wired</t>
-        </is>
-      </c>
-      <c r="G117" s="7" t="inlineStr"/>
-    </row>
-    <row r="118">
-      <c r="A118" s="5" t="inlineStr">
-        <is>
-          <t>Anthropic Claude</t>
-        </is>
-      </c>
-      <c r="B118" s="5" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="C118" s="5" t="inlineStr">
-        <is>
-          <t>Insight quality tier (recommendation copy)</t>
-        </is>
-      </c>
-      <c r="D118" s="5" t="inlineStr">
-        <is>
-          <t>ANTHROPIC_API_KEY (+ CONTENT_MODEL)</t>
-        </is>
-      </c>
-      <c r="E118" s="5" t="inlineStr">
-        <is>
-          <t>console.anthropic.com</t>
-        </is>
-      </c>
-      <c r="F118" s="6" t="inlineStr">
-        <is>
-          <t>✅ Wired</t>
-        </is>
-      </c>
-      <c r="G118" s="7" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="5" t="inlineStr">
         <is>
-          <t>Ollama</t>
+          <t>Supabase</t>
         </is>
       </c>
       <c r="B119" s="5" t="inlineStr">
         <is>
-          <t>AI / local</t>
+          <t>Core / DB</t>
         </is>
       </c>
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>CRO agent runs on-prem — privacy (data stays with business)</t>
+          <t>Events (funnel/returns) + cohorts + insights + Auth + RLS</t>
         </is>
       </c>
       <c r="D119" s="5" t="inlineStr">
         <is>
-          <t>OLLAMA_BASE_URL / OLLAMA_MODEL</t>
+          <t>NEXT_PUBLIC_SUPABASE_URL / _ANON_KEY / SUPABASE_SERVICE_ROLE_KEY</t>
         </is>
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t>ollama.com</t>
+          <t>supabase.com</t>
         </is>
       </c>
       <c r="F119" s="6" t="inlineStr">
@@ -4181,27 +4185,27 @@
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
-          <t>HELIX tag (JS snippet)</t>
+          <t>Anthropic Claude</t>
         </is>
       </c>
       <c r="B120" s="5" t="inlineStr">
         <is>
-          <t>Data source</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="C120" s="5" t="inlineStr">
         <is>
-          <t>First-party funnel + return events (embed on site)</t>
+          <t>Insight quality tier (recommendation copy)</t>
         </is>
       </c>
       <c r="D120" s="5" t="inlineStr">
         <is>
-          <t>public/helix-tag.js -&gt; /api/collect</t>
+          <t>ANTHROPIC_API_KEY (+ CONTENT_MODEL)</t>
         </is>
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t>internal</t>
+          <t>console.anthropic.com</t>
         </is>
       </c>
       <c r="F120" s="6" t="inlineStr">
@@ -4214,32 +4218,32 @@
     <row r="121">
       <c r="A121" s="5" t="inlineStr">
         <is>
-          <t>Microsoft Clarity</t>
+          <t>Ollama</t>
         </is>
       </c>
       <c r="B121" s="5" t="inlineStr">
         <is>
-          <t>Data source</t>
+          <t>AI / local</t>
         </is>
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>Heatmaps / session replay / funnels (FREE)</t>
+          <t>CRO agent runs on-prem — privacy (data stays with business)</t>
         </is>
       </c>
       <c r="D121" s="5" t="inlineStr">
         <is>
-          <t>Clarity API token (connector)</t>
+          <t>OLLAMA_BASE_URL / OLLAMA_MODEL</t>
         </is>
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t>clarity.microsoft.com</t>
+          <t>ollama.com</t>
         </is>
       </c>
       <c r="F121" s="6" t="inlineStr">
         <is>
-          <t>🔧 Planned</t>
+          <t>✅ Wired</t>
         </is>
       </c>
       <c r="G121" s="7" t="inlineStr"/>
@@ -4247,7 +4251,7 @@
     <row r="122">
       <c r="A122" s="5" t="inlineStr">
         <is>
-          <t>Google Analytics (GA4)</t>
+          <t>HELIX tag (JS snippet)</t>
         </is>
       </c>
       <c r="B122" s="5" t="inlineStr">
@@ -4257,22 +4261,22 @@
       </c>
       <c r="C122" s="5" t="inlineStr">
         <is>
-          <t>Traffic + conversion metrics</t>
+          <t>First-party funnel + return events (embed on site)</t>
         </is>
       </c>
       <c r="D122" s="5" t="inlineStr">
         <is>
-          <t>GOOGLE_OAUTH_* (reuse dashboards)</t>
+          <t>public/helix-tag.js -&gt; /api/collect</t>
         </is>
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t>console.cloud.google.com</t>
+          <t>internal</t>
         </is>
       </c>
       <c r="F122" s="6" t="inlineStr">
         <is>
-          <t>🔧 Planned</t>
+          <t>✅ Wired</t>
         </is>
       </c>
       <c r="G122" s="7" t="inlineStr"/>
@@ -4280,7 +4284,7 @@
     <row r="123">
       <c r="A123" s="5" t="inlineStr">
         <is>
-          <t>Mixpanel / Amplitude / PostHog</t>
+          <t>Microsoft Clarity</t>
         </is>
       </c>
       <c r="B123" s="5" t="inlineStr">
@@ -4290,22 +4294,22 @@
       </c>
       <c r="C123" s="5" t="inlineStr">
         <is>
-          <t>Retention / cohorts (optional, BYO)</t>
+          <t>Heatmaps / session replay / funnels (FREE)</t>
         </is>
       </c>
       <c r="D123" s="5" t="inlineStr">
         <is>
-          <t>API key per tool (connector)</t>
+          <t>Clarity API token (connector)</t>
         </is>
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t>each tool</t>
+          <t>clarity.microsoft.com</t>
         </is>
       </c>
       <c r="F123" s="6" t="inlineStr">
         <is>
-          <t>⚪ BYO</t>
+          <t>🔧 Planned</t>
         </is>
       </c>
       <c r="G123" s="7" t="inlineStr"/>
@@ -4313,32 +4317,32 @@
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
-          <t>WhatsApp Cloud API</t>
+          <t>Google Analytics (GA4)</t>
         </is>
       </c>
       <c r="B124" s="5" t="inlineStr">
         <is>
-          <t>Channel</t>
+          <t>Data source</t>
         </is>
       </c>
       <c r="C124" s="5" t="inlineStr">
         <is>
-          <t>Doctor digest + INBOUND bot (/api/whatsapp) + number linking via bot_links</t>
+          <t>Traffic + conversion metrics</t>
         </is>
       </c>
       <c r="D124" s="5" t="inlineStr">
         <is>
-          <t>WHATSAPP_TOKEN / WHATSAPP_PHONE_ID</t>
+          <t>GOOGLE_OAUTH_* (reuse dashboards)</t>
         </is>
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t>developers.facebook.com</t>
+          <t>console.cloud.google.com</t>
         </is>
       </c>
       <c r="F124" s="6" t="inlineStr">
         <is>
-          <t>✅ Wired</t>
+          <t>🔧 Planned</t>
         </is>
       </c>
       <c r="G124" s="7" t="inlineStr"/>
@@ -4346,32 +4350,32 @@
     <row r="125">
       <c r="A125" s="5" t="inlineStr">
         <is>
-          <t>Telegram Bot</t>
+          <t>Mixpanel / Amplitude / PostHog</t>
         </is>
       </c>
       <c r="B125" s="5" t="inlineStr">
         <is>
-          <t>Channel</t>
+          <t>Data source</t>
         </is>
       </c>
       <c r="C125" s="5" t="inlineStr">
         <is>
-          <t>Doctor digest + inbound actions (/api/bot)</t>
+          <t>Retention / cohorts (optional, BYO)</t>
         </is>
       </c>
       <c r="D125" s="5" t="inlineStr">
         <is>
-          <t>TELEGRAM_BOT_TOKEN</t>
+          <t>API key per tool (connector)</t>
         </is>
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t>@BotFather</t>
+          <t>each tool</t>
         </is>
       </c>
       <c r="F125" s="6" t="inlineStr">
         <is>
-          <t>✅ Wired</t>
+          <t>⚪ BYO</t>
         </is>
       </c>
       <c r="G125" s="7" t="inlineStr"/>
@@ -4379,7 +4383,7 @@
     <row r="126">
       <c r="A126" s="5" t="inlineStr">
         <is>
-          <t>Email (Resend)</t>
+          <t>WhatsApp Cloud API</t>
         </is>
       </c>
       <c r="B126" s="5" t="inlineStr">
@@ -4389,17 +4393,17 @@
       </c>
       <c r="C126" s="5" t="inlineStr">
         <is>
-          <t>Digest / report delivery</t>
+          <t>Doctor digest + INBOUND bot (/api/whatsapp) + number linking via bot_links</t>
         </is>
       </c>
       <c r="D126" s="5" t="inlineStr">
         <is>
-          <t>RESEND_API_KEY / EMAIL_FROM</t>
+          <t>WHATSAPP_TOKEN / WHATSAPP_PHONE_ID</t>
         </is>
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t>resend.com</t>
+          <t>developers.facebook.com</t>
         </is>
       </c>
       <c r="F126" s="6" t="inlineStr">
@@ -4412,32 +4416,32 @@
     <row r="127">
       <c r="A127" s="5" t="inlineStr">
         <is>
-          <t>HELIX OPS (reuse)</t>
+          <t>Telegram Bot</t>
         </is>
       </c>
       <c r="B127" s="5" t="inlineStr">
         <is>
-          <t>Cross-product</t>
+          <t>Channel</t>
         </is>
       </c>
       <c r="C127" s="5" t="inlineStr">
         <is>
-          <t>Execute the FIX — Landing / A-B / Campaigns / win-back</t>
+          <t>Doctor digest + inbound actions (/api/bot)</t>
         </is>
       </c>
       <c r="D127" s="5" t="inlineStr">
         <is>
-          <t>internal (same ecosystem)</t>
+          <t>TELEGRAM_BOT_TOKEN</t>
         </is>
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t>internal</t>
+          <t>@BotFather</t>
         </is>
       </c>
       <c r="F127" s="6" t="inlineStr">
         <is>
-          <t>🔧 Planned</t>
+          <t>✅ Wired</t>
         </is>
       </c>
       <c r="G127" s="7" t="inlineStr"/>
@@ -4445,27 +4449,27 @@
     <row r="128">
       <c r="A128" s="5" t="inlineStr">
         <is>
-          <t>HELIX DASHBOARDS export</t>
+          <t>Email (Resend)</t>
         </is>
       </c>
       <c r="B128" s="5" t="inlineStr">
         <is>
-          <t>Cross-product</t>
+          <t>Channel</t>
         </is>
       </c>
       <c r="C128" s="5" t="inlineStr">
         <is>
-          <t>Push CRO/funnel/retention metrics to super-dashboard</t>
+          <t>Digest / report delivery</t>
         </is>
       </c>
       <c r="D128" s="5" t="inlineStr">
         <is>
-          <t>EXPORT_SECRET (/api/export/growth-metrics)</t>
+          <t>RESEND_API_KEY / EMAIL_FROM</t>
         </is>
       </c>
       <c r="E128" s="5" t="inlineStr">
         <is>
-          <t>self-chosen</t>
+          <t>resend.com</t>
         </is>
       </c>
       <c r="F128" s="6" t="inlineStr">
@@ -4478,32 +4482,32 @@
     <row r="129">
       <c r="A129" s="5" t="inlineStr">
         <is>
-          <t>Cron secret</t>
+          <t>HELIX OPS (reuse)</t>
         </is>
       </c>
       <c r="B129" s="5" t="inlineStr">
         <is>
-          <t>Infra</t>
+          <t>Cross-product</t>
         </is>
       </c>
       <c r="C129" s="5" t="inlineStr">
         <is>
-          <t>Autonomous loop (measure-&gt;fix-&gt;re-measure)</t>
+          <t>Execute the FIX — Landing / A-B / Campaigns / win-back</t>
         </is>
       </c>
       <c r="D129" s="5" t="inlineStr">
         <is>
-          <t>CRON_SECRET</t>
+          <t>internal (same ecosystem)</t>
         </is>
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t>self-chosen</t>
+          <t>internal</t>
         </is>
       </c>
       <c r="F129" s="6" t="inlineStr">
         <is>
-          <t>✅ Wired</t>
+          <t>🔧 Planned</t>
         </is>
       </c>
       <c r="G129" s="7" t="inlineStr"/>
@@ -4511,100 +4515,166 @@
     <row r="130">
       <c r="A130" s="5" t="inlineStr">
         <is>
+          <t>HELIX DASHBOARDS export</t>
+        </is>
+      </c>
+      <c r="B130" s="5" t="inlineStr">
+        <is>
+          <t>Cross-product</t>
+        </is>
+      </c>
+      <c r="C130" s="5" t="inlineStr">
+        <is>
+          <t>Push CRO/funnel/retention metrics to super-dashboard</t>
+        </is>
+      </c>
+      <c r="D130" s="5" t="inlineStr">
+        <is>
+          <t>EXPORT_SECRET (/api/export/growth-metrics)</t>
+        </is>
+      </c>
+      <c r="E130" s="5" t="inlineStr">
+        <is>
+          <t>self-chosen</t>
+        </is>
+      </c>
+      <c r="F130" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G130" s="7" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="5" t="inlineStr">
+        <is>
+          <t>Cron secret</t>
+        </is>
+      </c>
+      <c r="B131" s="5" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="C131" s="5" t="inlineStr">
+        <is>
+          <t>Autonomous loop (measure-&gt;fix-&gt;re-measure)</t>
+        </is>
+      </c>
+      <c r="D131" s="5" t="inlineStr">
+        <is>
+          <t>CRON_SECRET</t>
+        </is>
+      </c>
+      <c r="E131" s="5" t="inlineStr">
+        <is>
+          <t>self-chosen</t>
+        </is>
+      </c>
+      <c r="F131" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G131" s="7" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="5" t="inlineStr">
+        <is>
           <t>Vercel</t>
         </is>
       </c>
-      <c r="B130" s="5" t="inlineStr">
+      <c r="B132" s="5" t="inlineStr">
         <is>
           <t>Infra</t>
         </is>
       </c>
-      <c r="C130" s="5" t="inlineStr">
+      <c r="C132" s="5" t="inlineStr">
         <is>
           <t>Hosting + Cron</t>
         </is>
       </c>
-      <c r="D130" s="5" t="inlineStr">
+      <c r="D132" s="5" t="inlineStr">
         <is>
           <t>git push (Helix-growth-doctor)</t>
         </is>
       </c>
-      <c r="E130" s="5" t="inlineStr">
+      <c r="E132" s="5" t="inlineStr">
         <is>
           <t>vercel.com</t>
         </is>
       </c>
-      <c r="F130" s="6" t="inlineStr">
+      <c r="F132" s="6" t="inlineStr">
         <is>
           <t>✅ Core</t>
         </is>
       </c>
-      <c r="G130" s="7" t="inlineStr"/>
-    </row>
-    <row r="131">
-      <c r="A131" t="inlineStr">
-        <is>
-          <t>### NEWLY-DISCOVERED / CORRECTED (git audit 04.08.2026) — see product sheets:</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" t="inlineStr">
-        <is>
-          <t>SDR: +Upstash Redis, +Lifecycle Schedule. Not-in-code: Instagram DM, Lusha/Hunter, Bright Data, Tavily/Exa, RB2B.</t>
-        </is>
-      </c>
+      <c r="G132" s="7" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>OPS: +Slack/Discord/WordPress/Lemmy/Twitch/Kick/MeWe/Dribbble, +Google Ads, +Outbrain, +Radar/Perf ingest. Meta Ads/HeyGen/D-ID -&gt; Wired. Typefully &amp; ElevenLabs -&gt; not-in-code.</t>
+          <t>### NEWLY-DISCOVERED / CORRECTED (git audit 04.08.2026) — see product sheets:</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Rank: +WordPress/Webhook publishers, +Wikidata/Wikipedia, +Dashboards export. Firecrawl -&gt; not-in-code (uses BrightData).</t>
+          <t>SDR: +Upstash Redis, +Lifecycle Schedule. Not-in-code: Instagram DM, Lusha/Hunter, Bright Data, Tavily/Exa, RB2B.</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>GEO Landing: +Wikipedia. Not-in-code (other apps): DataForSEO, Serper, GSC, Dicebear, Webhook secrets.</t>
+          <t>OPS: +Slack/Discord/WordPress/Lemmy/Twitch/Kick/MeWe/Dribbble, +Google Ads, +Outbrain, +Radar/Perf ingest. Meta Ads/HeyGen/D-ID -&gt; Wired. Typefully &amp; ElevenLabs -&gt; not-in-code.</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Dashboards: +HELIX SDR connector. Rav-Messer/ActiveTrail/InforU -&gt; Wired. Metrics ingest is PULL (CRON_SECRET).</t>
+          <t>Rank: +WordPress/Webhook publishers, +Wikidata/Wikipedia, +Dashboards export. Firecrawl -&gt; not-in-code (uses BrightData).</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Growth Doctor: +WhatsApp Templates registration. Cron secret -&gt; Planned (env only).</t>
+          <t>GEO Landing: +Wikipedia. Not-in-code (other apps): DataForSEO, Serper, GSC, Dicebear, Webhook secrets.</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
+          <t>Dashboards: +HELIX SDR connector. Rav-Messer/ActiveTrail/InforU -&gt; Wired. Metrics ingest is PULL (CRON_SECRET).</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Growth Doctor: +WhatsApp Templates registration. Cron secret -&gt; Planned (env only).</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
           <t>STAGE: +Google/LinkedIn OAuth login, +Scheduled email cron.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A67:G67"/>
-    <mergeCell ref="A91:G91"/>
+    <mergeCell ref="A93:G93"/>
+    <mergeCell ref="A69:G69"/>
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="A48:G48"/>
+    <mergeCell ref="A101:G101"/>
     <mergeCell ref="A25:G25"/>
-    <mergeCell ref="A99:G99"/>
   </mergeCells>
   <dataValidations count="6">
     <dataValidation sqref="G6:G23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>

<commit_message>
feat(free-tools): content tool (analyze/build/email) + email gate + nav section
- /free-tools/content: 3-mode Claude tool — post DNA analysis, post builder,
  email write/rewrite (HE+EN). API /api/content-tool (claude-sonnet-5).
- Email gate: /api/content-lead persists to Supabase (content_leads) + Resend
  notify; enforced server-side (/api/content-tool 403 without a valid email).
- Header: new "בדיקות חינם" dropdown (GEO + readiness + content); existing GEO
  & readiness links kept in place. Hamburger breakpoint 768→1279 so the 7-item
  nav never wraps.
- docs/content_leads.sql (run once); connections tracker updated.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCTS/HELIX-external-connections.xlsx
+++ b/PRODUCTS/HELIX-external-connections.xlsx
@@ -13,14 +13,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HELIX SEO-GEO BOT" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GEO Landing Page" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readiness Landing" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HELIX CRM" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HELIX STAGE" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HELIX Dashboards" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Channels matrix" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shared accounts" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup order" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HELIX Growth Doctor" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HELIX Account Portal" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Tool Landing" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HELIX CRM" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HELIX STAGE" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HELIX Dashboards" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Channels matrix" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shared accounts" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup order" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HELIX Growth Doctor" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HELIX Account Portal" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -676,7 +677,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G140"/>
+  <dimension ref="A1:G141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2682,7 +2683,6 @@
       </c>
       <c r="G67" s="7" t="inlineStr"/>
     </row>
-    <row r="68"/>
     <row r="69">
       <c r="A69" s="13" t="inlineStr">
         <is>
@@ -3420,7 +3420,6 @@
       </c>
       <c r="G91" s="7" t="inlineStr"/>
     </row>
-    <row r="92"/>
     <row r="93">
       <c r="A93" s="14" t="inlineStr">
         <is>
@@ -3630,7 +3629,6 @@
       </c>
       <c r="G99" s="7" t="inlineStr"/>
     </row>
-    <row r="100"/>
     <row r="101">
       <c r="A101" s="15" t="inlineStr">
         <is>
@@ -4104,7 +4102,6 @@
       </c>
       <c r="G115" s="7" t="inlineStr"/>
     </row>
-    <row r="116"/>
     <row r="117">
       <c r="A117" s="15" t="inlineStr">
         <is>
@@ -4664,6 +4661,13 @@
       <c r="A140" t="inlineStr">
         <is>
           <t>STAGE: +Google/LinkedIn OAuth login, +Scheduled email cron.</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Content Tool (/free-tools/content) — NEW 09.08.2026: Anthropic (analyze/build/email HE+EN) + Supabase content_leads (⚠️ להריץ docs/content_leads.sql + env ב-Vercel) + Resend notify + email gate (נאכף בשרת). שוכפל ל-OPS Performance: Content DNA + Post Builder + Email.</t>
         </is>
       </c>
     </row>
@@ -4706,6 +4710,752 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>HELIX Dashboards (Product 02)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Service / Channel</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Connect (token / OAuth / webhook / env)</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>Where to get it</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>Connected?</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Supabase</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Core / DB</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Widgets, dashboards, connector tokens (encrypted) + Auth</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>NEXT_PUBLIC_SUPABASE_URL / _ANON_KEY / SUPABASE_SERVICE_ROLE_KEY</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>supabase.com</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Anthropic Claude</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Narrate metrics + daily digest text</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>ANTHROPIC_API_KEY (+ CONTENT_MODEL)</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>console.anthropic.com</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Ollama</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>AI / local</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Local narration/classify — cost lever</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>OLLAMA_BASE_URL / OLLAMA_MODEL</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>ollama.com</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Google Analytics (GA4)</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Data source</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Traffic metrics into dashboards</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>GOOGLE_OAUTH_CLIENT_ID / _SECRET / _REDIRECT_URI</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>console.cloud.google.com</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Stripe</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Data source</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Revenue / MRR metrics</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Stripe connector token (encrypted via SECRETS_KEY)</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>dashboard.stripe.com/apikeys</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Plausible Analytics</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Data source</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Privacy analytics metrics</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Plausible API key (connector)</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>plausible.io</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Meta / Facebook Insights</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Data source</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Social page/post insights</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>FB_APP_ID / FB_APP_SECRET</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>developers.facebook.com</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Metrics ingest (from HELIX products)</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Data source</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Receives pushed metrics (SDR/OPS/SEO-GEO → dashboards)</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>PULL via /api/connectors/sync + /api/cron/sync (CRON_SECRET) — no HELIX_DASHBOARDS_KEY</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Email (Resend)</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Deliver daily digest / reports</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>RESEND_API_KEY / EMAIL_FROM</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>resend.com</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Telegram Bot</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Digest delivery + bot</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>TELEGRAM_BOT_TOKEN</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>@BotFather</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>WhatsApp Cloud API</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Digest delivery (with chart image) + INBOUND bot (/api/whatsapp) + number linking via bot_links</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>WHATSAPP_TOKEN / WHATSAPP_PHONE_ID</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>developers.facebook.com</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Secrets / Cron</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Encrypt connector tokens + schedule digests</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>SECRETS_KEY / CRON_SECRET</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>self-chosen</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Vercel</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Hosting + Cron</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>git push (HELIX-DASHBOARDS)</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>vercel.com</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>✅ Core</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Shopify</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Data source</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>E-commerce metrics into dashboards (sales / orders / AOV)</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Shopify Admin API token + shop domain (connector, encrypted via SECRETS_KEY)</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>&lt;shop&gt;.myshopify.com → Admin API</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Mailchimp</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Data source</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Email list metrics (subscribers / unsubscribes)</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Mailchimp API key (connector, encrypted)</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>mailchimp.com → Account → API keys</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>HELIX OPS (campaign A/B)</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Data source / cross-product</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Pull campaign A/B metrics (impressions/views/clicks/variants per channel) into dashboards</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>base_url + Export Secret + OPS workspace id (connector)</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>internal (helix-ops /api/export/campaign-metrics)</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Rav-Messer (Responder)</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Data source</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Israeli email/SMS marketing metrics (list subscribers) into dashboards</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>User Key (+ optional Secret) — connector, encrypted</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>support@responder.co.il / 03-717-7777</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>verify endpoint schema</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>ActiveTrail</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Data source</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Israeli email/SMS marketing metrics (contacts/subscribers) into dashboards</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>API key (connector, encrypted)</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>ActiveTrail account → Settings → API</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>verify endpoint schema</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>InforU</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Data source</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Israeli SMS/email marketing metrics (contact groups) into dashboards</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>API key (connector, encrypted)</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>InforU account → API</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>verify endpoint schema</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>HELIX SDR (connector)</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Data source</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Pulls SDR metrics</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>SDR_EXPORT_URL + EXPORT_SECRET</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="G3:G15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"not yet,in progress,done"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5061,7 +5811,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5242,13 +5992,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:D55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6022,6 +6772,82 @@
       <c r="D50" s="5" t="inlineStr">
         <is>
           <t>schedule the digest</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="26" t="inlineStr">
+        <is>
+          <t>Content Tool Landing</t>
+        </is>
+      </c>
+      <c r="B51" s="30" t="inlineStr"/>
+      <c r="C51" s="5" t="inlineStr"/>
+      <c r="D51" s="5" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="29" t="inlineStr"/>
+      <c r="B52" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>Anthropic Claude key</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>the tool itself (analyze / build post / write+rewrite email)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="29" t="inlineStr"/>
+      <c r="B53" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>Supabase + run docs/content_leads.sql</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>capture the gate emails (persist leads)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="29" t="inlineStr"/>
+      <c r="B54" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>Resend (RESEND_NOTIFY_TO)</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>get notified on each new lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="29" t="inlineStr"/>
+      <c r="B55" s="30" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>— verify SUPABASE_URL / SUPABASE_SERVICE_KEY on Vercel</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>so captured emails actually persist</t>
         </is>
       </c>
     </row>
@@ -6038,7 +6864,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6599,7 +7425,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11825,6 +12651,278 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="38" t="inlineStr">
+        <is>
+          <t>בדיקת תוכן בחינם (Content Tool) — /free-tools/content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="39" t="inlineStr">
+        <is>
+          <t>⚠️ Deploy: static export → /api/* מחזיר 404 → הכלי עובד רק מ-deploy של Vercel (שרת). שער מייל חובה לפני שימוש (נאכף בשרת).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="40" t="inlineStr">
+        <is>
+          <t>Service / Channel</t>
+        </is>
+      </c>
+      <c r="B3" s="40" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C3" s="40" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="D3" s="40" t="inlineStr">
+        <is>
+          <t>Connect (token / OAuth / webhook / env)</t>
+        </is>
+      </c>
+      <c r="E3" s="40" t="inlineStr">
+        <is>
+          <t>Where to get it</t>
+        </is>
+      </c>
+      <c r="F3" s="40" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G3" s="40" t="inlineStr">
+        <is>
+          <t>Connected?</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="24" t="inlineStr">
+        <is>
+          <t>Anthropic Claude</t>
+        </is>
+      </c>
+      <c r="B4" s="24" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="C4" s="24" t="inlineStr">
+        <is>
+          <t>ניתוח פוסטים (DNA) + בניית פוסטים + כתיבה/שכתוב מיילים HE/EN (lib/content-tool.ts)</t>
+        </is>
+      </c>
+      <c r="D4" s="24" t="inlineStr">
+        <is>
+          <t>ANTHROPIC_API_KEY (model claude-sonnet-5)</t>
+        </is>
+      </c>
+      <c r="E4" s="24" t="inlineStr">
+        <is>
+          <t>console.anthropic.com</t>
+        </is>
+      </c>
+      <c r="F4" s="24" t="inlineStr">
+        <is>
+          <t>🔧 Coded — needs key</t>
+        </is>
+      </c>
+      <c r="G4" s="24" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="24" t="inlineStr">
+        <is>
+          <t>Supabase (content_leads)</t>
+        </is>
+      </c>
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>Core / DB</t>
+        </is>
+      </c>
+      <c r="C5" s="24" t="inlineStr">
+        <is>
+          <t>לכידת המייל משער הכניסה (recordContentLead, source=content)</t>
+        </is>
+      </c>
+      <c r="D5" s="24" t="inlineStr">
+        <is>
+          <t>SUPABASE_URL / SUPABASE_SERVICE_KEY</t>
+        </is>
+      </c>
+      <c r="E5" s="24" t="inlineStr">
+        <is>
+          <t>supabase.com</t>
+        </is>
+      </c>
+      <c r="F5" s="24" t="inlineStr">
+        <is>
+          <t>🔧 צריך לטפל: הרץ docs/content_leads.sql + ודא env ב-Vercel</t>
+        </is>
+      </c>
+      <c r="G5" s="24" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="24" t="inlineStr">
+        <is>
+          <t>Email (Resend)</t>
+        </is>
+      </c>
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="C6" s="24" t="inlineStr">
+        <is>
+          <t>התראה על ליד חדש (best-effort — לא חוסם unlock)</t>
+        </is>
+      </c>
+      <c r="D6" s="24" t="inlineStr">
+        <is>
+          <t>RESEND_API_KEY / RESEND_NOTIFY_TO</t>
+        </is>
+      </c>
+      <c r="E6" s="24" t="inlineStr">
+        <is>
+          <t>resend.com</t>
+        </is>
+      </c>
+      <c r="F6" s="24" t="inlineStr">
+        <is>
+          <t>✅ Wired (best-effort)</t>
+        </is>
+      </c>
+      <c r="G6" s="24" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="24" t="inlineStr">
+        <is>
+          <t>Email gate</t>
+        </is>
+      </c>
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>Gate / Lead</t>
+        </is>
+      </c>
+      <c r="C7" s="24" t="inlineStr">
+        <is>
+          <t>חובה מייל תקין כדי להשתמש — נאכף גם בשרת (/api/content-tool → 403 בלי מייל); נזכר ב-localStorage</t>
+        </is>
+      </c>
+      <c r="D7" s="24" t="inlineStr">
+        <is>
+          <t>internal (/api/content-lead)</t>
+        </is>
+      </c>
+      <c r="E7" s="24" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F7" s="24" t="inlineStr">
+        <is>
+          <t>✅ Wired</t>
+        </is>
+      </c>
+      <c r="G7" s="24" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="24" t="inlineStr">
+        <is>
+          <t>Vercel</t>
+        </is>
+      </c>
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="C8" s="24" t="inlineStr">
+        <is>
+          <t>Hosting (helix website repo)</t>
+        </is>
+      </c>
+      <c r="D8" s="24" t="inlineStr">
+        <is>
+          <t>git push vercel master</t>
+        </is>
+      </c>
+      <c r="E8" s="24" t="inlineStr">
+        <is>
+          <t>vercel.com</t>
+        </is>
+      </c>
+      <c r="F8" s="24" t="inlineStr">
+        <is>
+          <t>✅ Core</t>
+        </is>
+      </c>
+      <c r="G8" s="24" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="24" t="inlineStr">
+        <is>
+          <t>HELIX OPS (mirror)</t>
+        </is>
+      </c>
+      <c r="B9" s="24" t="inlineStr">
+        <is>
+          <t>Cross-product</t>
+        </is>
+      </c>
+      <c r="C9" s="24" t="inlineStr">
+        <is>
+          <t>אותם 2 פיצ׳רים כפנימיים ב-OPS: Post Builder + Email writer (+ Content DNA) ב-Performance grid</t>
+        </is>
+      </c>
+      <c r="D9" s="24" t="inlineStr">
+        <is>
+          <t>ANTHROPIC_API_KEY (של OPS)</t>
+        </is>
+      </c>
+      <c r="E9" s="24" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F9" s="24" t="inlineStr">
+        <is>
+          <t>✅ Code</t>
+        </is>
+      </c>
+      <c r="G9" s="24" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -12132,7 +13230,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12434,750 +13532,4 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="15" t="inlineStr">
-        <is>
-          <t>HELIX Dashboards (Product 02)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>Service / Channel</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>Purpose</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>Connect (token / OAuth / webhook / env)</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>Where to get it</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>Connected?</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>Supabase</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>Core / DB</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>Widgets, dashboards, connector tokens (encrypted) + Auth</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>NEXT_PUBLIC_SUPABASE_URL / _ANON_KEY / SUPABASE_SERVICE_ROLE_KEY</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>supabase.com</t>
-        </is>
-      </c>
-      <c r="F3" s="6" t="inlineStr">
-        <is>
-          <t>✅ Wired</t>
-        </is>
-      </c>
-      <c r="G3" s="7" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>Anthropic Claude</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>Narrate metrics + daily digest text</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>ANTHROPIC_API_KEY (+ CONTENT_MODEL)</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>console.anthropic.com</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>✅ Wired</t>
-        </is>
-      </c>
-      <c r="G4" s="7" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Ollama</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>AI / local</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Local narration/classify — cost lever</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>OLLAMA_BASE_URL / OLLAMA_MODEL</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>ollama.com</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>✅ Wired</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Google Analytics (GA4)</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Data source</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Traffic metrics into dashboards</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>GOOGLE_OAUTH_CLIENT_ID / _SECRET / _REDIRECT_URI</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>console.cloud.google.com</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>✅ Wired</t>
-        </is>
-      </c>
-      <c r="G6" s="7" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Stripe</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Data source</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Revenue / MRR metrics</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Stripe connector token (encrypted via SECRETS_KEY)</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>dashboard.stripe.com/apikeys</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>✅ Wired</t>
-        </is>
-      </c>
-      <c r="G7" s="7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Plausible Analytics</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Data source</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Privacy analytics metrics</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Plausible API key (connector)</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>plausible.io</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>✅ Wired</t>
-        </is>
-      </c>
-      <c r="G8" s="7" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Meta / Facebook Insights</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Data source</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Social page/post insights</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>FB_APP_ID / FB_APP_SECRET</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>developers.facebook.com</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>✅ Wired</t>
-        </is>
-      </c>
-      <c r="G9" s="7" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Metrics ingest (from HELIX products)</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Data source</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Receives pushed metrics (SDR/OPS/SEO-GEO → dashboards)</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>PULL via /api/connectors/sync + /api/cron/sync (CRON_SECRET) — no HELIX_DASHBOARDS_KEY</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>internal</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>✅ Wired</t>
-        </is>
-      </c>
-      <c r="G10" s="7" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Email (Resend)</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Channel</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Deliver daily digest / reports</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>RESEND_API_KEY / EMAIL_FROM</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>resend.com</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>✅ Wired</t>
-        </is>
-      </c>
-      <c r="G11" s="7" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>Telegram Bot</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Channel</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Digest delivery + bot</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>TELEGRAM_BOT_TOKEN</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>@BotFather</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>✅ Wired</t>
-        </is>
-      </c>
-      <c r="G12" s="7" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>WhatsApp Cloud API</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Channel</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Digest delivery (with chart image) + INBOUND bot (/api/whatsapp) + number linking via bot_links</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>WHATSAPP_TOKEN / WHATSAPP_PHONE_ID</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>developers.facebook.com</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>✅ Wired</t>
-        </is>
-      </c>
-      <c r="G13" s="7" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>Secrets / Cron</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>Infra</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Encrypt connector tokens + schedule digests</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>SECRETS_KEY / CRON_SECRET</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>self-chosen</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>✅ Wired</t>
-        </is>
-      </c>
-      <c r="G14" s="7" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>Vercel</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Infra</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Hosting + Cron</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>git push (HELIX-DASHBOARDS)</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>vercel.com</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>✅ Core</t>
-        </is>
-      </c>
-      <c r="G15" s="7" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>Shopify</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Data source</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>E-commerce metrics into dashboards (sales / orders / AOV)</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Shopify Admin API token + shop domain (connector, encrypted via SECRETS_KEY)</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>&lt;shop&gt;.myshopify.com → Admin API</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>✅ Wired</t>
-        </is>
-      </c>
-      <c r="G16" s="7" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>Mailchimp</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>Data source</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>Email list metrics (subscribers / unsubscribes)</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>Mailchimp API key (connector, encrypted)</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>mailchimp.com → Account → API keys</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="inlineStr">
-        <is>
-          <t>✅ Wired</t>
-        </is>
-      </c>
-      <c r="G17" s="7" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>HELIX OPS (campaign A/B)</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Data source / cross-product</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Pull campaign A/B metrics (impressions/views/clicks/variants per channel) into dashboards</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>base_url + Export Secret + OPS workspace id (connector)</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>internal (helix-ops /api/export/campaign-metrics)</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="inlineStr">
-        <is>
-          <t>✅ Wired</t>
-        </is>
-      </c>
-      <c r="G18" s="7" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>Rav-Messer (Responder)</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>Data source</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Israeli email/SMS marketing metrics (list subscribers) into dashboards</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>User Key (+ optional Secret) — connector, encrypted</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>support@responder.co.il / 03-717-7777</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>✅ Wired</t>
-        </is>
-      </c>
-      <c r="G19" s="7" t="inlineStr">
-        <is>
-          <t>verify endpoint schema</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>ActiveTrail</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>Data source</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Israeli email/SMS marketing metrics (contacts/subscribers) into dashboards</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>API key (connector, encrypted)</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>ActiveTrail account → Settings → API</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr">
-        <is>
-          <t>✅ Wired</t>
-        </is>
-      </c>
-      <c r="G20" s="7" t="inlineStr">
-        <is>
-          <t>verify endpoint schema</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>InforU</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>Data source</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>Israeli SMS/email marketing metrics (contact groups) into dashboards</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>API key (connector, encrypted)</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>InforU account → API</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr">
-        <is>
-          <t>✅ Wired</t>
-        </is>
-      </c>
-      <c r="G21" s="7" t="inlineStr">
-        <is>
-          <t>verify endpoint schema</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>HELIX SDR (connector)</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>Data source</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Pulls SDR metrics</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>SDR_EXPORT_URL + EXPORT_SECRET</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>internal</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr">
-        <is>
-          <t>✅ Wired</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
-  </mergeCells>
-  <dataValidations count="1">
-    <dataValidation sqref="G3:G15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"not yet,in progress,done"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(free-tools): free-usage quota (4) then upgrade to HELIX OPS
- Meter build/email uses per email in Supabase (content_tool_usage); analysis
  stays free & unmetered. FREE_LIMIT=4.
- /api/content-tool enforces the quota (402 quota_exceeded) and returns
  `remaining`; adds a `status` probe. /api/content-lead returns remaining on unlock.
- Tool shows "נותרו X מתוך 4" and swaps to an upgrade-to-HELIX-OPS panel
  (my.helix.co.il) once the quota is spent.
- docs/content_tool_usage.sql (run once); connections tracker updated.
- Degrades to unlimited when Supabase isn't configured (localhost).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCTS/HELIX-external-connections.xlsx
+++ b/PRODUCTS/HELIX-external-connections.xlsx
@@ -4667,7 +4667,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Content Tool (/free-tools/content) — NEW 09.08.2026: Anthropic (analyze/build/email HE+EN) + Supabase content_leads (⚠️ להריץ docs/content_leads.sql + env ב-Vercel) + Resend notify + email gate (נאכף בשרת). שוכפל ל-OPS Performance: Content DNA + Post Builder + Email.</t>
+          <t>Content Tool (/free-tools/content) — NEW 09.08.2026: Anthropic (analyze/build/email HE+EN) + Supabase content_leads (⚠️ להריץ docs/content_leads.sql + env ב-Vercel) + Resend notify + email gate (נאכף בשרת). שוכפל ל-OPS Performance: Content DNA + Post Builder + Email + paywall: 4 שימושים חינמיים (build/email) → שדרוג ל-HELIX OPS (docs/content_tool_usage.sql).</t>
         </is>
       </c>
     </row>
@@ -12651,7 +12651,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -12783,32 +12783,32 @@
     <row r="6">
       <c r="A6" s="24" t="inlineStr">
         <is>
-          <t>Email (Resend)</t>
+          <t>Supabase (content_tool_usage)</t>
         </is>
       </c>
       <c r="B6" s="24" t="inlineStr">
         <is>
-          <t>Channel</t>
+          <t>Metering / Paywall</t>
         </is>
       </c>
       <c r="C6" s="24" t="inlineStr">
         <is>
-          <t>התראה על ליד חדש (best-effort — לא חוסם unlock)</t>
+          <t>4 שימושים חינמיים (build+email); אח״כ שדרוג ל-HELIX OPS. ניתוח (DNA) חינם ללא הגבלה</t>
         </is>
       </c>
       <c r="D6" s="24" t="inlineStr">
         <is>
-          <t>RESEND_API_KEY / RESEND_NOTIFY_TO</t>
+          <t>SUPABASE_URL / SUPABASE_SERVICE_KEY</t>
         </is>
       </c>
       <c r="E6" s="24" t="inlineStr">
         <is>
-          <t>resend.com</t>
+          <t>supabase.com</t>
         </is>
       </c>
       <c r="F6" s="24" t="inlineStr">
         <is>
-          <t>✅ Wired (best-effort)</t>
+          <t>🔧 צריך לטפל: הרץ docs/content_tool_usage.sql</t>
         </is>
       </c>
       <c r="G6" s="24" t="inlineStr"/>
@@ -12816,32 +12816,32 @@
     <row r="7">
       <c r="A7" s="24" t="inlineStr">
         <is>
-          <t>Email gate</t>
+          <t>Email (Resend)</t>
         </is>
       </c>
       <c r="B7" s="24" t="inlineStr">
         <is>
-          <t>Gate / Lead</t>
+          <t>Channel</t>
         </is>
       </c>
       <c r="C7" s="24" t="inlineStr">
         <is>
-          <t>חובה מייל תקין כדי להשתמש — נאכף גם בשרת (/api/content-tool → 403 בלי מייל); נזכר ב-localStorage</t>
+          <t>התראה על ליד חדש (best-effort — לא חוסם unlock)</t>
         </is>
       </c>
       <c r="D7" s="24" t="inlineStr">
         <is>
-          <t>internal (/api/content-lead)</t>
+          <t>RESEND_API_KEY / RESEND_NOTIFY_TO</t>
         </is>
       </c>
       <c r="E7" s="24" t="inlineStr">
         <is>
-          <t>internal</t>
+          <t>resend.com</t>
         </is>
       </c>
       <c r="F7" s="24" t="inlineStr">
         <is>
-          <t>✅ Wired</t>
+          <t>✅ Wired (best-effort)</t>
         </is>
       </c>
       <c r="G7" s="24" t="inlineStr"/>
@@ -12849,32 +12849,32 @@
     <row r="8">
       <c r="A8" s="24" t="inlineStr">
         <is>
-          <t>Vercel</t>
+          <t>Email gate</t>
         </is>
       </c>
       <c r="B8" s="24" t="inlineStr">
         <is>
-          <t>Infra</t>
+          <t>Gate / Lead</t>
         </is>
       </c>
       <c r="C8" s="24" t="inlineStr">
         <is>
-          <t>Hosting (helix website repo)</t>
+          <t>חובה מייל תקין כדי להשתמש — נאכף גם בשרת (/api/content-tool → 403 בלי מייל); נזכר ב-localStorage</t>
         </is>
       </c>
       <c r="D8" s="24" t="inlineStr">
         <is>
-          <t>git push vercel master</t>
+          <t>internal (/api/content-lead)</t>
         </is>
       </c>
       <c r="E8" s="24" t="inlineStr">
         <is>
-          <t>vercel.com</t>
+          <t>internal</t>
         </is>
       </c>
       <c r="F8" s="24" t="inlineStr">
         <is>
-          <t>✅ Core</t>
+          <t>✅ Wired</t>
         </is>
       </c>
       <c r="G8" s="24" t="inlineStr"/>
@@ -12882,35 +12882,68 @@
     <row r="9">
       <c r="A9" s="24" t="inlineStr">
         <is>
+          <t>Vercel</t>
+        </is>
+      </c>
+      <c r="B9" s="24" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="C9" s="24" t="inlineStr">
+        <is>
+          <t>Hosting (helix website repo)</t>
+        </is>
+      </c>
+      <c r="D9" s="24" t="inlineStr">
+        <is>
+          <t>git push vercel master</t>
+        </is>
+      </c>
+      <c r="E9" s="24" t="inlineStr">
+        <is>
+          <t>vercel.com</t>
+        </is>
+      </c>
+      <c r="F9" s="24" t="inlineStr">
+        <is>
+          <t>✅ Core</t>
+        </is>
+      </c>
+      <c r="G9" s="24" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="24" t="inlineStr">
+        <is>
           <t>HELIX OPS (mirror)</t>
         </is>
       </c>
-      <c r="B9" s="24" t="inlineStr">
+      <c r="B10" s="24" t="inlineStr">
         <is>
           <t>Cross-product</t>
         </is>
       </c>
-      <c r="C9" s="24" t="inlineStr">
+      <c r="C10" s="24" t="inlineStr">
         <is>
           <t>אותם 2 פיצ׳רים כפנימיים ב-OPS: Post Builder + Email writer (+ Content DNA) ב-Performance grid</t>
         </is>
       </c>
-      <c r="D9" s="24" t="inlineStr">
+      <c r="D10" s="24" t="inlineStr">
         <is>
           <t>ANTHROPIC_API_KEY (של OPS)</t>
         </is>
       </c>
-      <c r="E9" s="24" t="inlineStr">
+      <c r="E10" s="24" t="inlineStr">
         <is>
           <t>internal</t>
         </is>
       </c>
-      <c r="F9" s="24" t="inlineStr">
+      <c r="F10" s="24" t="inlineStr">
         <is>
           <t>✅ Code</t>
         </is>
       </c>
-      <c r="G9" s="24" t="inlineStr"/>
+      <c r="G10" s="24" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs(status): content tools + free-tool paywall — done & to-complete
- Performance status (docx): +content-tools row in "מה נעשה"; dated 09.08 update
  block with the website free tool, email gate, 4-use quota, and the pending
  Supabase SQL / Vercel env steps.
- Connections (xlsx): OPS sheet +content-tools row; Content Tool Landing sheet
  already flags content_leads.sql + content_tool_usage.sql as "🔧 צריך לטפל".

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCTS/HELIX-external-connections.xlsx
+++ b/PRODUCTS/HELIX-external-connections.xlsx
@@ -9353,7 +9353,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -10762,6 +10762,39 @@
           <t>needs v19+v20 SQL</t>
         </is>
       </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Content tools (DNA / Post / Email)</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>AI / Content</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>3 כרטיסים בגריד Performance: ניתוח DNA של פוסטים, בניית פוסט (HE/EN), כתיבה/שכתוב מיילים HE/EN. מקביל לכלי החינמי באתר.</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>ANTHROPIC_API_KEY (קיים)</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t>✅ Code</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
docs(growth-doctor): reflect autonomy switch across product page + specs + xlsx
- products-data.ts: new "מתג אוטונומיה" feature + control/safety FAQ
- 07-growth-doctor.docx: new autonomy-layer section
- HELIX SOFTWARES REVIEW PAGES.docx: growth-doctor autonomy note
- HELIX-external-connections.xlsx: autonomy_settings status row (run autonomy.sql)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCTS/HELIX-external-connections.xlsx
+++ b/PRODUCTS/HELIX-external-connections.xlsx
@@ -6870,7 +6870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -7417,6 +7417,43 @@
       <c r="F17" s="6" t="inlineStr">
         <is>
           <t>✅ Wired</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Autonomy switch (autonomy_settings)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Capability / DB</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>מתג 3-מצבי advisor/approve/autopilot — ה-CTA של תובנות פועל בפועל</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>supabase/autonomy.sql (autonomy_settings + autonomy_actions)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>internal — no external key</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>🔧 Coded — run migration</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>⚠️ הרץ autonomy.sql</t>
         </is>
       </c>
     </row>
@@ -10794,7 +10831,6 @@
           <t>✅ Code</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
docs(sdr): reflect autonomy switch across product page + specs + xlsx
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCTS/HELIX-external-connections.xlsx
+++ b/PRODUCTS/HELIX-external-connections.xlsx
@@ -8162,7 +8162,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -9368,6 +9368,43 @@
       <c r="F37" s="6" t="inlineStr">
         <is>
           <t>✅ Wired</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Autonomy switch (autonomy_settings)</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Capability / DB</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>מתג 3-מצבי לפנייה — autopilot כ-opt-in מפורש; בסיס=מאשר</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>supabase/autonomy.sql</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>internal — no external key</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>🔧 Coded — run migration</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>⚠️ הרץ autonomy.sql</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(ops): reflect autonomy switch across product page + specs + xlsx
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCTS/HELIX-external-connections.xlsx
+++ b/PRODUCTS/HELIX-external-connections.xlsx
@@ -9427,7 +9427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -10866,6 +10866,43 @@
       <c r="F43" s="6" t="inlineStr">
         <is>
           <t>✅ Code</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Autonomy switch (autonomy_settings)</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Capability / DB</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>מתג 3-מצבי חוצה-מודולים; radar autopilot כ-opt-in</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>supabase/autonomy.sql</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>internal — no external key</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>🔧 Coded — run migration</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>⚠️ הרץ autonomy.sql</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(rank): reflect autonomy publish-behind-switch across page + specs + xlsx
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCTS/HELIX-external-connections.xlsx
+++ b/PRODUCTS/HELIX-external-connections.xlsx
@@ -10925,7 +10925,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -11634,6 +11634,43 @@
       <c r="F22" s="6" t="inlineStr">
         <is>
           <t>✅ Wired</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Autonomy switch (autonomy_settings)</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Capability / DB</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>פרסום-חי ל-CMS מאחורי מתג (site-scoped); autopilot כ-opt-in</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>supabase/autonomy.sql</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>internal — no external key</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>🔧 Coded — run migration</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>⚠️ הרץ autonomy.sql</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(crm): reflect autonomy stalled-deal detector across CRM spec + xlsx
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCTS/HELIX-external-connections.xlsx
+++ b/PRODUCTS/HELIX-external-connections.xlsx
@@ -13136,7 +13136,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -13435,6 +13435,43 @@
       <c r="G10" s="24" t="inlineStr">
         <is>
           <t>STAGE כבר יש</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Autonomy switch (autonomy_settings)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Capability / DB</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>עסקה מידרדרת→פעולה; crm.next_step internal (autopilot ללא ack)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>supabase/autonomy.sql</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>internal — no external key</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>🔧 Coded — run migration</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>⚠️ הרץ autonomy.sql</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(dashboards): reflect slipping-KPI alert + hub foundation across page + specs + xlsx
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCTS/HELIX-external-connections.xlsx
+++ b/PRODUCTS/HELIX-external-connections.xlsx
@@ -4710,7 +4710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5434,6 +5434,43 @@
       <c r="F22" s="6" t="inlineStr">
         <is>
           <t>✅ Wired</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Autonomy switch (autonomy_settings)</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Capability / DB</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>slipping-KPI בדייג'סט + hub foundation (dash.cross_act בהמשך)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>supabase/autonomy.sql</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>internal — no external key</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>🔧 Coded — run migration</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>⚠️ הרץ autonomy.sql</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(autonomy): Phase 4 cross-product dispatch — spec + hub page + specs + xlsx env
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCTS/HELIX-external-connections.xlsx
+++ b/PRODUCTS/HELIX-external-connections.xlsx
@@ -4710,7 +4710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5471,6 +5471,43 @@
       <c r="G23" t="inlineStr">
         <is>
           <t>⚠️ הרץ autonomy.sql</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Cross-act dispatch (Phase 4)</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Integration / outbound</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>מ-hub מפעיל טריגר במוצר אחר כשמדד מידרדר (dash.cross_act)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>env: GROWTH_DOCTOR_URL + CROSS_ACT_SECRET</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>self (product URLs)</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>🔧 Coded — set env to enable</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>⚪ optional — no-op ללא env</t>
         </is>
       </c>
     </row>
@@ -6907,7 +6944,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -7491,6 +7528,43 @@
       <c r="G18" t="inlineStr">
         <is>
           <t>⚠️ הרץ autonomy.sql</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Cross-act trigger endpoint (Phase 4)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Integration / inbound</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>POST /api/act/trigger — hub מפעיל אבחון+פעולה דרך המתג</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>env: CROSS_ACT_SECRET</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>🔧 Coded — set secret to enable</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>⚪ optional</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(autonomy): Phase 4 triggers for OPS/SDR/Rank — specs + xlsx env rows
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCTS/HELIX-external-connections.xlsx
+++ b/PRODUCTS/HELIX-external-connections.xlsx
@@ -8273,7 +8273,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -9516,6 +9516,43 @@
       <c r="G38" t="inlineStr">
         <is>
           <t>⚠️ הרץ autonomy.sql</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Cross-act trigger endpoint (Phase 4)</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Integration / inbound</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>POST /api/act/trigger — hub מפעיל את הליבה דרך המתג של המוצר</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>env: CROSS_ACT_SECRET</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>🔧 Coded — set secret to enable</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>⚪ optional</t>
         </is>
       </c>
     </row>
@@ -9538,7 +9575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -11014,6 +11051,43 @@
       <c r="G44" t="inlineStr">
         <is>
           <t>⚠️ הרץ autonomy.sql</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Cross-act trigger endpoint (Phase 4)</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Integration / inbound</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>POST /api/act/trigger — hub מפעיל את הליבה דרך המתג של המוצר</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>env: CROSS_ACT_SECRET</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>🔧 Coded — set secret to enable</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>⚪ optional</t>
         </is>
       </c>
     </row>
@@ -11036,7 +11110,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -11782,6 +11856,43 @@
       <c r="G23" t="inlineStr">
         <is>
           <t>⚠️ הרץ autonomy.sql</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Cross-act trigger endpoint (Phase 4)</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Integration / inbound</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>POST /api/act/trigger — hub מפעיל את הליבה דרך המתג של המוצר</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>env: CROSS_ACT_SECRET</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>🔧 Coded — set secret to enable</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>⚪ optional</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(autonomy): sync switch UI across product pages + specs + xlsx
Adds the settings-screen mention to 5 product pages, a UI section to each product
docx, and a settings-page-route row to each xlsx product sheet — closing the doc
gap for the switch UI work.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCTS/HELIX-external-connections.xlsx
+++ b/PRODUCTS/HELIX-external-connections.xlsx
@@ -4710,7 +4710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5508,6 +5508,43 @@
       <c r="G24" t="inlineStr">
         <is>
           <t>⚪ optional — no-op ללא env</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Autonomy switch UI (settings page)</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>מסך הגדרות לבחירת מצב per-feature: /settings — פקד 3-מצבי עם אפקט, checkbox risk_ack</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>in-app</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>✅ Built</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -6944,7 +6981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -7565,6 +7602,43 @@
       <c r="G19" t="inlineStr">
         <is>
           <t>⚪ optional</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Autonomy switch UI (settings page)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>מסך הגדרות לבחירת מצב per-feature: panel on home — פקד 3-מצבי עם אפקט, checkbox risk_ack</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>in-app</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>✅ Built</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -8273,7 +8347,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -9553,6 +9627,43 @@
       <c r="G39" t="inlineStr">
         <is>
           <t>⚪ optional</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Autonomy switch UI (settings page)</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>מסך הגדרות לבחירת מצב per-feature: /autonomy — פקד 3-מצבי עם אפקט, checkbox risk_ack</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>in-app</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>✅ Built</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -9575,7 +9686,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -11088,6 +11199,43 @@
       <c r="G45" t="inlineStr">
         <is>
           <t>⚪ optional</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Autonomy switch UI (settings page)</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>מסך הגדרות לבחירת מצב per-feature: /[locale]/autonomy — פקד 3-מצבי עם אפקט, checkbox risk_ack</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>in-app</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>✅ Built</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -11110,7 +11258,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -11893,6 +12041,43 @@
       <c r="G24" t="inlineStr">
         <is>
           <t>⚪ optional</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Autonomy switch UI (settings page)</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>מסך הגדרות לבחירת מצב per-feature: /autonomy (per-site) — פקד 3-מצבי עם אפקט, checkbox risk_ack</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>in-app</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>✅ Built</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -13358,7 +13543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -13694,6 +13879,43 @@
       <c r="G11" t="inlineStr">
         <is>
           <t>⚠️ הרץ autonomy.sql</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Autonomy switch UI (settings page)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>מסך הגדרות לבחירת מצב per-feature: /dashboard/crm/autonomy — פקד 3-מצבי עם אפקט, checkbox risk_ack</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>in-app</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>✅ Built</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(products): competitive analysis — HELIX Ecosystem vs Wix Symphony
Wix Symphony (AI-agent SMB platform) is a near-mirror of the ecosystem thesis:
AI CRM hub + specialized agents + Maestro orchestrator + separate workspaces
+ approval workflows + credit pricing. Validates direction. Key moves: build a
HELIX Maestro orchestrator (our gap), market as "AI team of agents", lean on
moats (Hebrew/RTL, WhatsApp-native, standalone/not-website-locked, on-prem
privacy, per-action autonomy). Notes gaps Symphony reveals (Finance/Design agents).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCTS/HELIX-external-connections.xlsx
+++ b/PRODUCTS/HELIX-external-connections.xlsx
@@ -22,6 +22,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup order" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HELIX Growth Doctor" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HELIX Account Portal" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HELIX MEETING" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -31,7 +32,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -82,6 +83,15 @@
       <i val="1"/>
       <color rgb="00B45309"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0010B981"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="16">
@@ -232,7 +242,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -312,6 +322,9 @@
     <xf numFmtId="0" fontId="8" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -677,7 +690,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G141"/>
+  <dimension ref="A1:G158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -699,10 +712,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Status: ✅ Wired = live in code  ·  🔧 Planned/Partial = in spec, not fully wired  ·  ⚪ Optional/BYO  |  Update 04.08.2026: WhatsApp inbound bot + number→account linking wired across Dashboards/Growth-Doctor/SDR/OPS/Rank; Rank WhatsApp 🔧→✅.  |  Full git re-audit 04.08.2026: statuses corrected vs actual code; newly-found integrations appended per product sheet + addendum below.</t>
-        </is>
-      </c>
-    </row>
+          <t>Status: ✅ Wired = live in code  ·  🔧 Planned/Partial = in spec, not fully wired  ·  ⚪ Optional/BYO  |  Update 04.08.2026: WhatsApp inbound bot + number→account linking wired across Dashboards/Growth-Doctor/SDR/OPS/GEO; GEO WhatsApp 🔧→✅.  |  Full git re-audit 04.08.2026: statuses corrected vs actual code; newly-found integrations appended per product sheet + addendum below.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1341,6 +1355,7 @@
       </c>
       <c r="G23" s="7" t="inlineStr"/>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="10" t="inlineStr">
         <is>
@@ -2045,6 +2060,7 @@
       </c>
       <c r="G46" s="7" t="inlineStr"/>
     </row>
+    <row r="47"/>
     <row r="48">
       <c r="A48" s="12" t="inlineStr">
         <is>
@@ -2683,6 +2699,7 @@
       </c>
       <c r="G67" s="7" t="inlineStr"/>
     </row>
+    <row r="68"/>
     <row r="69">
       <c r="A69" s="13" t="inlineStr">
         <is>
@@ -3420,6 +3437,7 @@
       </c>
       <c r="G91" s="7" t="inlineStr"/>
     </row>
+    <row r="92"/>
     <row r="93">
       <c r="A93" s="14" t="inlineStr">
         <is>
@@ -3629,6 +3647,7 @@
       </c>
       <c r="G99" s="7" t="inlineStr"/>
     </row>
+    <row r="100"/>
     <row r="101">
       <c r="A101" s="15" t="inlineStr">
         <is>
@@ -4102,6 +4121,7 @@
       </c>
       <c r="G115" s="7" t="inlineStr"/>
     </row>
+    <row r="116"/>
     <row r="117">
       <c r="A117" s="15" t="inlineStr">
         <is>
@@ -4668,6 +4688,499 @@
       <c r="A141" t="inlineStr">
         <is>
           <t>Content Tool (/free-tools/content) — NEW 09.08.2026: Anthropic (analyze/build/email HE+EN) + Supabase content_leads (⚠️ להריץ docs/content_leads.sql + env ב-Vercel) + Resend notify + email gate (נאכף בשרת). שוכפל ל-OPS Performance: Content DNA + Post Builder + Email + paywall: 4 שימושים חינמיים (build/email) → שדרוג ל-HELIX OPS (docs/content_tool_usage.sql).</t>
+        </is>
+      </c>
+    </row>
+    <row r="142"/>
+    <row r="143">
+      <c r="A143" s="41" t="inlineStr">
+        <is>
+          <t>HELIX MEETING AND RECORDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="42" t="inlineStr">
+        <is>
+          <t>Service / Channel</t>
+        </is>
+      </c>
+      <c r="B144" s="42" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C144" s="42" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="D144" s="42" t="inlineStr">
+        <is>
+          <t>Connect (token / OAuth / webhook)</t>
+        </is>
+      </c>
+      <c r="E144" s="42" t="inlineStr">
+        <is>
+          <t>Where to get it</t>
+        </is>
+      </c>
+      <c r="F144" s="42" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G144" s="42" t="inlineStr">
+        <is>
+          <t>Connected?</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Supabase</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Core / DB</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>meetings/transcripts/moments/bookings + autonomy</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>NEXT_PUBLIC_SUPABASE_URL / SERVICE_ROLE</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>supabase.com</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>🔧 Coded — run schema.sql</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Anthropic Claude</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Summary + action items + 6-signal engine + follow-up draft</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>ANTHROPIC_API_KEY</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>console.anthropic.com</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>✅ Wired (code)</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>ivrit.ai Whisper (self-host)</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>AI / STT</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Hebrew transcription (whisper-large-v3) on HELIX servers</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>IVRIT_WHISPER_URL / IVRIT_WHISPER_TOKEN</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>huggingface.co/ivrit-ai (self-host VM/GPU)</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>🔧 Coded — needs server</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Supabase Storage (meeting-audio)</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Storage</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Store uploaded audio before transcription</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>bucket "meeting-audio"</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>supabase.com</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>🔧 Create bucket</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Vexa (self-host)</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Capture / bot</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Meeting bot join Zoom/Meet/Teams (mode B)</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>VEXA_BASE_URL / VEXA_API_KEY</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>vexa.ai (self-host, Apache 2.0)</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>⬜ Not in code (planned)</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>WhatsApp Cloud API</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Voice-note capture (mode D) + follow-up + approve buttons</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>reuse SDR Meta app + Graph /media</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>developers.facebook.com</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>🔧 Reuse SDR + add /media</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Telegram Bot</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Voice-note capture (mode D) + approve</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>reuse SDR TELEGRAM_BOT_TOKEN</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>@BotFather</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>🔧 Reuse SDR + add voice</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Email (send-as-user)</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Send follow-up in user voice (Gmail/Outlook OAuth)</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>reuse plug-nexus send-email-via-user</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>🔧 Wire execute→send</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Google Calendar</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Scheduling</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Booking page availability + bot joins booked meeting</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>GOOGLE_OAUTH_* (reuse plug-nexus)</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>console.cloud.google.com</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>🔧 Reuse plug-nexus fns</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>PLUG extension (tabCapture)</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Capture</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Tab-audio capture in browser (mode A)</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>extension build</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>⬜ Not in code (planned)</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Meetily (desktop, MIT)</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Capture</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Local system-audio desktop app (mode C)</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>self-host / fork</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>meetily.ai</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>⬜ Planned (phase 3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Cross-product act (SDR/CRM/OPS/GEO)</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Push signals as leads/tasks/content</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>CROSS_ACT_SECRET → POST /api/act/trigger</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>🔧 Coded seam — wire</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Autonomy switch (autonomy_settings)</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Capability / DB</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Per-signal advisor/approve/autopilot</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>supabase/schema.sql</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>internal — no external key</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>✅ Coded (copy-in)</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Vercel</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Hosting</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>git push</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>vercel.com</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>⬜ New repo — add</t>
         </is>
       </c>
     </row>
@@ -5567,7 +6080,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5620,6 +6133,11 @@
           <t>HELIX Growth Doctor</t>
         </is>
       </c>
+      <c r="I1" s="18" t="inlineStr">
+        <is>
+          <t>HELIX MEETING</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="18" t="inlineStr">
@@ -5654,6 +6172,11 @@
           <t>✅</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>🔧</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="18" t="inlineStr">
@@ -5690,6 +6213,11 @@
       <c r="H3" s="19" t="inlineStr">
         <is>
           <t>✅</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>🔧</t>
         </is>
       </c>
     </row>
@@ -5796,6 +6324,11 @@
           <t>✅</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="18" t="inlineStr">
@@ -5896,6 +6429,11 @@
       <c r="H12" s="19" t="inlineStr">
         <is>
           <t>✅</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -7672,6 +8210,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="37" t="inlineStr">
         <is>
@@ -8335,6 +8874,529 @@
         </is>
       </c>
       <c r="G22" s="37" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="43" t="inlineStr">
+        <is>
+          <t>HELIX MEETING AND RECORDING (Product 10 · repo helix/helix-meeting)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Status: ✅ Wired · 🔧 Coded/needs infra · ⬜ Not in code yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="42" t="inlineStr">
+        <is>
+          <t>Service / Channel</t>
+        </is>
+      </c>
+      <c r="B4" s="42" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C4" s="42" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="D4" s="42" t="inlineStr">
+        <is>
+          <t>Connect (token / OAuth / webhook)</t>
+        </is>
+      </c>
+      <c r="E4" s="42" t="inlineStr">
+        <is>
+          <t>Where to get it</t>
+        </is>
+      </c>
+      <c r="F4" s="42" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G4" s="42" t="inlineStr">
+        <is>
+          <t>Connected?</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Supabase</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Core / DB</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>meetings/transcripts/moments/bookings + autonomy</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>NEXT_PUBLIC_SUPABASE_URL / SERVICE_ROLE</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>supabase.com</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>🔧 Coded — run schema.sql</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Anthropic Claude</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Summary + action items + 6-signal engine + follow-up draft</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>ANTHROPIC_API_KEY</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>console.anthropic.com</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>✅ Wired (code)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ivrit.ai Whisper (self-host)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>AI / STT</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Hebrew transcription (whisper-large-v3) on HELIX servers</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>IVRIT_WHISPER_URL / IVRIT_WHISPER_TOKEN</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>huggingface.co/ivrit-ai (self-host VM/GPU)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>🔧 Coded — needs server</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Supabase Storage (meeting-audio)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Storage</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Store uploaded audio before transcription</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>bucket "meeting-audio"</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>supabase.com</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>🔧 Create bucket</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Vexa (self-host)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Capture / bot</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Meeting bot join Zoom/Meet/Teams (mode B)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>VEXA_BASE_URL / VEXA_API_KEY</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>vexa.ai (self-host, Apache 2.0)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>⬜ Not in code (planned)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>WhatsApp Cloud API</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Voice-note capture (mode D) + follow-up + approve buttons</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>reuse SDR Meta app + Graph /media</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>developers.facebook.com</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>🔧 Reuse SDR + add /media</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Telegram Bot</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Voice-note capture (mode D) + approve</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>reuse SDR TELEGRAM_BOT_TOKEN</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>@BotFather</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>🔧 Reuse SDR + add voice</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Email (send-as-user)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Send follow-up in user voice (Gmail/Outlook OAuth)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>reuse plug-nexus send-email-via-user</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>🔧 Wire execute→send</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Google Calendar</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Scheduling</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Booking page availability + bot joins booked meeting</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>GOOGLE_OAUTH_* (reuse plug-nexus)</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>console.cloud.google.com</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>🔧 Reuse plug-nexus fns</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>PLUG extension (tabCapture)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Capture</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Tab-audio capture in browser (mode A)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>extension build</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>⬜ Not in code (planned)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Meetily (desktop, MIT)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Capture</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Local system-audio desktop app (mode C)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>self-host / fork</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>meetily.ai</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>⬜ Planned (phase 3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Cross-product act (SDR/CRM/OPS/GEO)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Push signals as leads/tasks/content</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>CROSS_ACT_SECRET → POST /api/act/trigger</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>🔧 Coded seam — wire</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Autonomy switch (autonomy_settings)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Capability / DB</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Per-signal advisor/approve/autopilot</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>supabase/schema.sql</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>internal — no external key</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>✅ Coded (copy-in)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Vercel</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Hosting</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>git push</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>vercel.com</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>⬜ New repo — add</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>